<commit_message>
Daily Amazon price update
</commit_message>
<xml_diff>
--- a/amazon_products.xlsx
+++ b/amazon_products.xlsx
@@ -7061,12 +7061,12 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Acer Smartchoice Aspire One, Intel Core Celeron N4500, Office 2024 + M365 Basic, 12GB LPDDR4X / 256GB SSD, 14.0"/35.56cm TN HD Display, Win 11 Home, Pure Silver, 1.3KG, A114-45, Thin and Light Laptop</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="B317" t="inlineStr"/>
       <c r="C317" t="n">
-        <v>32990</v>
+        <v>44999</v>
       </c>
       <c r="D317" t="inlineStr">
         <is>
@@ -7075,7 +7075,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Acer Smartchoice Aspire One, Intel</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily Amazon price update - 2026-07-12
</commit_message>
<xml_diff>
--- a/amazon_products.xlsx
+++ b/amazon_products.xlsx
@@ -7061,12 +7061,12 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Acer Smartchoice Aspire One, Intel Core Celeron N4500, Office 2024 + M365 Basic, 12GB LPDDR4X / 512GB SSD, 14.0"/35.56cm TN HD Display, Win 11 Home, Pure Silver, 1.3KG, A114-45, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="B317" t="inlineStr"/>
       <c r="C317" t="n">
-        <v>44999</v>
+        <v>34990</v>
       </c>
       <c r="D317" t="inlineStr">
         <is>
@@ -7075,7 +7075,7 @@
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Acer Smartchoice Aspire One, Intel</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Daily Amazon price update - 2026-07-21
</commit_message>
<xml_diff>
--- a/amazon_products.xlsx
+++ b/amazon_products.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E344"/>
+  <dimension ref="A1:E352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2546,21 +2546,21 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Neo 13″</t>
+          <t>acer_travellite_thin_laptop_amd</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Neo 13″ Laptop with A18 Pro chip: Built for AI and Apple Intelligence, Liquid Retina Display, 8GB Unified Memory, 256GB SSD Storage, 1080p FaceTime HD Camera; Citrus</t>
+          <t>Acer TravelLite Thin Laptop AMD Ryzen 5 7430U (6-Core) 16GB RAM, 512GB SSD 14" Full HD Anti-Glare Display Privacy Shutter Windows 11 MS Office Metal Body 1.34Kg Black 30M Warranty</t>
         </is>
       </c>
       <c r="C102" t="inlineStr"/>
       <c r="D102" t="n">
-        <v>65000</v>
+        <v>52999</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -2572,16 +2572,16 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Neo 13″ Laptop with A18 Pro chip: Built for AI and Apple Intelligence, Liquid Retina Display, 8GB Unified Memory, 256GB SSD Storage, 1080p FaceTime HD Camera; Indigo</t>
+          <t>Apple 2026 MacBook Neo 13″ Laptop with A18 Pro chip: Built for AI and Apple Intelligence, Liquid Retina Display, 8GB Unified Memory, 256GB SSD Storage, 1080p FaceTime HD Camera; Citrus</t>
         </is>
       </c>
       <c r="C103" t="inlineStr"/>
       <c r="D103" t="n">
-        <v>67900</v>
+        <v>65000</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -2598,11 +2598,11 @@
       </c>
       <c r="C104" t="inlineStr"/>
       <c r="D104" t="n">
-        <v>65000</v>
+        <v>67900</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -2619,11 +2619,11 @@
       </c>
       <c r="C105" t="inlineStr"/>
       <c r="D105" t="n">
-        <v>65700</v>
+        <v>65000</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -2640,11 +2640,11 @@
       </c>
       <c r="C106" t="inlineStr"/>
       <c r="D106" t="n">
-        <v>65000</v>
+        <v>65700</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2665,7 @@
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2686,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -2698,7 +2698,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Neo 13″ Laptop with A18 Pro chip: Built for AI and Apple Intelligence, Liquid Retina Display, 8GB Unified Memory, 256GB SSD Storage, 1080p FaceTime HD Camera; Silver</t>
+          <t>Apple 2026 MacBook Neo 13″ Laptop with A18 Pro chip: Built for AI and Apple Intelligence, Liquid Retina Display, 8GB Unified Memory, 256GB SSD Storage, 1080p FaceTime HD Camera; Indigo</t>
         </is>
       </c>
       <c r="C109" t="inlineStr"/>
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -2745,11 +2745,11 @@
       </c>
       <c r="C111" t="inlineStr"/>
       <c r="D111" t="n">
-        <v>65700</v>
+        <v>65000</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -2766,11 +2766,11 @@
       </c>
       <c r="C112" t="inlineStr"/>
       <c r="D112" t="n">
-        <v>67900</v>
+        <v>65700</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -2787,11 +2787,11 @@
       </c>
       <c r="C113" t="inlineStr"/>
       <c r="D113" t="n">
-        <v>65000</v>
+        <v>67900</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -2808,11 +2808,11 @@
       </c>
       <c r="C114" t="inlineStr"/>
       <c r="D114" t="n">
-        <v>64990</v>
+        <v>65000</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -2829,11 +2829,11 @@
       </c>
       <c r="C115" t="inlineStr"/>
       <c r="D115" t="n">
-        <v>63990</v>
+        <v>64990</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -2875,28 +2875,28 @@
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Pro Laptop</t>
+          <t>Apple 2026 MacBook Neo 13″</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Pro Laptop with M5 Max chip with 18‑core CPU and 40‑core GPU: Built for AI, 41.05 cm (16.2″) Liquid Retina XDR Display, 48GB Unified Memory, 2TB SSD Storage; Space Black</t>
+          <t>Apple 2026 MacBook Neo 13″ Laptop with A18 Pro chip: Built for AI and Apple Intelligence, Liquid Retina Display, 8GB Unified Memory, 256GB SSD Storage, 1080p FaceTime HD Camera; Silver</t>
         </is>
       </c>
       <c r="C118" t="inlineStr"/>
       <c r="D118" t="n">
-        <v>499900</v>
+        <v>63990</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -2917,7 +2917,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -2938,7 +2938,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -2950,16 +2950,16 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Apple 2026 MacBook Pro Laptop with M5 Pro chip with 15‑core CPU and 16‑core GPU: Built for AI, 35.97 cm (14.2″) Liquid Retina XDR Display, 24GB Unified Memory, 1TB SSD Storage; Silver</t>
+          <t>Apple 2026 MacBook Pro Laptop with M5 Max chip with 18‑core CPU and 40‑core GPU: Built for AI, 41.05 cm (16.2″) Liquid Retina XDR Display, 48GB Unified Memory, 2TB SSD Storage; Space Black</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
       <c r="D121" t="n">
-        <v>234900</v>
+        <v>499900</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -2976,32 +2976,32 @@
       </c>
       <c r="C122" t="inlineStr"/>
       <c r="D122" t="n">
-        <v>227400</v>
+        <v>234900</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BrowseBook 14.1" FHD IPS Laptop</t>
+          <t>Apple 2026 MacBook Pro Laptop</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>BrowseBook 14.1" FHD IPS Laptop | Best Student &amp; Office Work Laptop | Celeron N4020 | 4GB RAM | 128GB SSD | Windows 11 | 38Wh | 1.3kg | Grey</t>
+          <t>Apple 2026 MacBook Pro Laptop with M5 Pro chip with 15‑core CPU and 16‑core GPU: Built for AI, 35.97 cm (14.2″) Liquid Retina XDR Display, 24GB Unified Memory, 1TB SSD Storage; Silver</t>
         </is>
       </c>
       <c r="C123" t="inlineStr"/>
       <c r="D123" t="n">
-        <v>13990</v>
+        <v>227400</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -3022,7 +3022,7 @@
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -3043,7 +3043,7 @@
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -3060,11 +3060,11 @@
       </c>
       <c r="C126" t="inlineStr"/>
       <c r="D126" t="n">
-        <v>20990</v>
+        <v>13990</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
@@ -3076,37 +3076,37 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>BrowseBook 14.1" FHD IPS Laptop | Best Student &amp; Office Work Laptop | Celeron N4020 | 8GB RAM | 256GB SSD | Windows 11 | 38Wh | 1.3kg | Grey</t>
+          <t>BrowseBook 14.1" FHD IPS Laptop | Best Student &amp; Office Work Laptop | Celeron N4020 | 4GB RAM | 128GB SSD | Windows 11 | 38Wh | 1.3kg | Grey</t>
         </is>
       </c>
       <c r="C127" t="inlineStr"/>
       <c r="D127" t="n">
-        <v>18990</v>
+        <v>20990</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Dell 15 (Previously Inspiron) Laptop,</t>
+          <t>BrowseBook 14.1" FHD IPS Laptop</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Dell 15 (Previously Inspiron) Laptop, 14th Gen Intel Core 3 100U Processor, 8GB DDR4, 512 SSD, 15.6" NT FHD 120Hz IPS AG 250 nit Display, Win 11 + Office H&amp;S 2024, Carbon Black, Thin &amp; Light- 1.63Kg</t>
+          <t>BrowseBook 14.1" FHD IPS Laptop | Best Student &amp; Office Work Laptop | Celeron N4020 | 8GB RAM | 256GB SSD | Windows 11 | 38Wh | 1.3kg | Grey</t>
         </is>
       </c>
       <c r="C128" t="inlineStr"/>
       <c r="D128" t="n">
-        <v>46490</v>
+        <v>18990</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -3118,16 +3118,16 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Dell 15 (Previously Inspiron) Laptop, 14th Gen Intel Core i3/Core 3 100U Processor, 8GB DDR4, 512 SSD, 15.6" FHD 120Hz IPS 250 nit Display, Win 11 + Office H&amp;S 2024, Carbon Black, Thin &amp; Light 1.63Kg</t>
+          <t>Dell 15 (Previously Inspiron) Laptop, 14th Gen Intel Core 3 100U Processor, 8GB DDR4, 512 SSD, 15.6" NT FHD 120Hz IPS AG 250 nit Display, Win 11 + Office H&amp;S 2024, Carbon Black, Thin &amp; Light- 1.63Kg</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
       <c r="D129" t="n">
-        <v>45490</v>
+        <v>46490</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -3144,11 +3144,11 @@
       </c>
       <c r="C130" t="inlineStr"/>
       <c r="D130" t="n">
-        <v>44990</v>
+        <v>45490</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -3169,7 +3169,7 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -3186,11 +3186,11 @@
       </c>
       <c r="C132" t="inlineStr"/>
       <c r="D132" t="n">
-        <v>45490</v>
+        <v>44990</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -3211,7 +3211,7 @@
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -3232,7 +3232,7 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -3249,11 +3249,11 @@
       </c>
       <c r="C135" t="inlineStr"/>
       <c r="D135" t="n">
-        <v>46490</v>
+        <v>45490</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -3270,116 +3270,116 @@
       </c>
       <c r="C136" t="inlineStr"/>
       <c r="D136" t="n">
-        <v>46990</v>
+        <v>46490</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>dell_15_(previously_inspiron)_laptop,</t>
+          <t>Dell 15 (Previously Inspiron) Laptop,</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Dell 15 (Previously Inspiron) Laptop, 14th Gen Intel Core i3/Core 3 100U Processor, 8GB, 512GB, Intel UHD Graphics, 15.6" FHD IPS 250nit Display, 12m Mcafee, Win 11 + MSO'24, Platinum Silver, 1.63kg</t>
+          <t>Dell 15 (Previously Inspiron) Laptop, 14th Gen Intel Core i3/Core 3 100U Processor, 8GB DDR4, 512 SSD, 15.6" FHD 120Hz IPS 250 nit Display, Win 11 + Office H&amp;S 2024, Carbon Black, Thin &amp; Light 1.63Kg</t>
         </is>
       </c>
       <c r="C137" t="inlineStr"/>
       <c r="D137" t="n">
-        <v>50490</v>
+        <v>46990</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Dell 15 (Previously Inspiron), 13th</t>
+          <t>dell_15_(previously_inspiron)_laptop,</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Dell 15 (Previously Inspiron), 13th Gen Intel Core i5-1334U (16GB RAM, 1TB SSD) FHD, Anti-Glare 15.6"/39.62cm, Windows 11 MSO'24, Silver, 1.62kg, 12 Month McAfee, Thin &amp; Light, Backlit Keyboard Laptop</t>
+          <t>Dell 15 (Previously Inspiron) Laptop, 14th Gen Intel Core i3/Core 3 100U Processor, 8GB, 512GB, Intel UHD Graphics, 15.6" FHD IPS 250nit Display, 12m Mcafee, Win 11 + MSO'24, Platinum Silver, 1.63kg</t>
         </is>
       </c>
       <c r="C138" t="inlineStr"/>
       <c r="D138" t="n">
-        <v>63990</v>
+        <v>50490</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Dell 15 AI Powered Laptop,</t>
+          <t>Dell 15 (Previously Inspiron), 13th</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Dell 15 AI Powered Laptop, Intel Core Ultra 5 225H, 8GB DDR5 RAM, 512GB SSD, 15.6" FHD Anti-Glare Display, Intel Arc Graphics, Standard Keyboard, Dedicated Copilot Key, Black, Win11 Home + MSO H&amp;S'24</t>
+          <t>Dell 15 (Previously Inspiron), 13th Gen Intel Core i5-1334U (16GB RAM, 1TB SSD) FHD, Anti-Glare 15.6"/39.62cm, Windows 11 MSO'24, Silver, 1.62kg, 12 Month McAfee, Thin &amp; Light, Backlit Keyboard Laptop</t>
         </is>
       </c>
       <c r="C139" t="inlineStr"/>
       <c r="D139" t="n">
-        <v>68990</v>
+        <v>63990</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>dell_15_ai_powered_laptop,</t>
+          <t>Dell 15 AI Powered Laptop,</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Dell 15 Ai Powered Laptop, Intel Core Ultra 7 255H, 16GB DDR5 RAM, 512GB SSD, 15.6" FHD Anti-Glare Display, Intel Arc Graphics, Backlit Keyboard, Dedicated Copilot Key, Silver, Win11 Home + MSO H&amp;S'24</t>
+          <t>Dell 15 AI Powered Laptop, Intel Core Ultra 5 225H, 8GB DDR5 RAM, 512GB SSD, 15.6" FHD Anti-Glare Display, Intel Arc Graphics, Standard Keyboard, Dedicated Copilot Key, Black, Win11 Home + MSO H&amp;S'24</t>
         </is>
       </c>
       <c r="C140" t="inlineStr"/>
       <c r="D140" t="n">
-        <v>103990</v>
+        <v>68990</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Dell 15 Smart Choice (Previously</t>
+          <t>dell_15_ai_powered_laptop,</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Dell 15 Smart Choice (Previously Inspiron), 13th Gen Intel Core i5-1334U (16GB RAM, 1TB SSD) FHD, 15.6"/39.62cm, Windows 11 MSO'24, Silver, 1.62kg, 12 Month McAfee, Backlit KB, Thin &amp; Light Laptop</t>
+          <t>Dell 15 Ai Powered Laptop, Intel Core Ultra 7 255H, 16GB DDR5 RAM, 512GB SSD, 15.6" FHD Anti-Glare Display, Intel Arc Graphics, Backlit Keyboard, Dedicated Copilot Key, Silver, Win11 Home + MSO H&amp;S'24</t>
         </is>
       </c>
       <c r="C141" t="inlineStr"/>
       <c r="D141" t="n">
-        <v>66990</v>
+        <v>103990</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -3396,11 +3396,11 @@
       </c>
       <c r="C142" t="inlineStr"/>
       <c r="D142" t="n">
-        <v>67990</v>
+        <v>66990</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -3421,7 +3421,7 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -3438,11 +3438,11 @@
       </c>
       <c r="C144" t="inlineStr"/>
       <c r="D144" t="n">
-        <v>69990</v>
+        <v>67990</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -3459,32 +3459,32 @@
       </c>
       <c r="C145" t="inlineStr"/>
       <c r="D145" t="n">
-        <v>67990</v>
+        <v>69990</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Dell 15, 13th Gen Intel</t>
+          <t>Dell 15 Smart Choice (Previously</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Dell 15, 13th Gen Intel Core i5-1334U (16GB DDR4, 512GB SSD) Anti-Glare FHD 15.6"/39.62cm, Windows 11, Microsoft Office Home 2024, Grey, 1.66kg, [Vostro 3530], 12 Month McAfee, Thin &amp; Light Laptop</t>
+          <t>Dell 15 Smart Choice (Previously Inspiron), 13th Gen Intel Core i5-1334U (16GB RAM, 1TB SSD) FHD, 15.6"/39.62cm, Windows 11 MSO'24, Silver, 1.62kg, 12 Month McAfee, Backlit KB, Thin &amp; Light Laptop</t>
         </is>
       </c>
       <c r="C146" t="inlineStr"/>
       <c r="D146" t="n">
-        <v>61490</v>
+        <v>67990</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-06-14</t>
         </is>
       </c>
     </row>
@@ -3501,32 +3501,32 @@
       </c>
       <c r="C147" t="inlineStr"/>
       <c r="D147" t="n">
-        <v>63490</v>
+        <v>61490</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Dell 15, AMD Ryzen 7-7730U,</t>
+          <t>Dell 15, 13th Gen Intel</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Dell 15, AMD Ryzen 7-7730U, 16GB DDR4, 512GB SSD, FHD, 15.6"/39.6cm, Windows 11, Microsoft Office Home 2024, Platinum Silver, 1.63Kg, [Dell 15], 120Hz 250nits, AMD Radeon Graphics,Thin &amp; Light, Laptop</t>
+          <t>Dell 15, 13th Gen Intel Core i5-1334U (16GB DDR4, 512GB SSD) Anti-Glare FHD 15.6"/39.62cm, Windows 11, Microsoft Office Home 2024, Grey, 1.66kg, [Vostro 3530], 12 Month McAfee, Thin &amp; Light Laptop</t>
         </is>
       </c>
       <c r="C148" t="inlineStr"/>
       <c r="D148" t="n">
-        <v>59957</v>
+        <v>63490</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -3543,116 +3543,116 @@
       </c>
       <c r="C149" t="inlineStr"/>
       <c r="D149" t="n">
-        <v>58490</v>
+        <v>59957</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Dell 15, Intel Core 3</t>
+          <t>Dell 15, AMD Ryzen 7-7730U,</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Dell 15, Intel Core 3 14th Gen-100U, 16GB DDR4, 512GB SSD, FHD IPS, 15.6"/39.62cm, Windows 11, Microsoft Office Home 2024, Carbon Black, 1.63Kg, Thin &amp; Light, Laptop Model NO - Dell 15 DCU5250</t>
+          <t>Dell 15, AMD Ryzen 7-7730U, 16GB DDR4, 512GB SSD, FHD, 15.6"/39.6cm, Windows 11, Microsoft Office Home 2024, Platinum Silver, 1.63Kg, [Dell 15], 120Hz 250nits, AMD Radeon Graphics,Thin &amp; Light, Laptop</t>
         </is>
       </c>
       <c r="C150" t="inlineStr"/>
       <c r="D150" t="n">
-        <v>51868</v>
+        <v>58490</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Dell 15, Intel Core i3/Core</t>
+          <t>Dell 15, Intel Core 3</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Dell 15, Intel Core i3/Core 3 14th Gen-100U, 16GB DDR4, 512GB SSD, FHD IPS, 15.6"/39.62cm, Windows 11, Microsoft Office Home 2024, Carbon Black, 1.63Kg, Thin &amp; Light, Laptop Model NO - Dell 15 DCU5250</t>
+          <t>Dell 15, Intel Core 3 14th Gen-100U, 16GB DDR4, 512GB SSD, FHD IPS, 15.6"/39.62cm, Windows 11, Microsoft Office Home 2024, Carbon Black, 1.63Kg, Thin &amp; Light, Laptop Model NO - Dell 15 DCU5250</t>
         </is>
       </c>
       <c r="C151" t="inlineStr"/>
       <c r="D151" t="n">
-        <v>48990</v>
+        <v>51868</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Dell 15, R5-7520U Processor, 8GB</t>
+          <t>Dell 15, Intel Core i3/Core</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Dell 15, R5-7520U Processor, 8GB LPDDR5 RAM, 512GB SSD, FHD 15.6"/39.62 cm Display, Windows 11, MSO'24, Carbon Black, 1.63kg, Standard Keyboard, 15 Month McAfee, Thin &amp; Light Laptop</t>
+          <t>Dell 15, Intel Core i3/Core 3 14th Gen-100U, 16GB DDR4, 512GB SSD, FHD IPS, 15.6"/39.62cm, Windows 11, Microsoft Office Home 2024, Carbon Black, 1.63Kg, Thin &amp; Light, Laptop Model NO - Dell 15 DCU5250</t>
         </is>
       </c>
       <c r="C152" t="inlineStr"/>
       <c r="D152" t="n">
-        <v>53990</v>
+        <v>48990</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>dell_g_series,_intel_core</t>
+          <t>Dell 15, R5-7520U Processor, 8GB</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Dell G Series, Intel Core i5-13450HX, 13th Gen, NVIDIA RTX 3050-6GB, 16GB, 512GB SSD, FHD, 15.6"/39.62cm, Windows 11, MSO'24, Dark Shadow Gray, 2.65KG, [G15-5530], Backlit Keyboard, Gaming Laptop</t>
+          <t>Dell 15, R5-7520U Processor, 8GB LPDDR5 RAM, 512GB SSD, FHD 15.6"/39.62 cm Display, Windows 11, MSO'24, Carbon Black, 1.63kg, Standard Keyboard, 15 Month McAfee, Thin &amp; Light Laptop</t>
         </is>
       </c>
       <c r="C153" t="inlineStr"/>
       <c r="D153" t="n">
-        <v>89990</v>
+        <v>53990</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Dell G15, 13th Gen Intel</t>
+          <t>dell_g_series,_intel_core</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Dell G15, 13th Gen Intel Core i5-13450HX Processor, NVIDIA RTX 3050-6GB, (16GB RAM 1TB SSD) FHD 15.6"/39.62 cm, Orange Backlit Keyboard, Win 11, MS Office'24, Dark Shadow Grey, 2.65Kg Gaming Laptop</t>
+          <t>Dell G Series, Intel Core i5-13450HX, 13th Gen, NVIDIA RTX 3050-6GB, 16GB, 512GB SSD, FHD, 15.6"/39.62cm, Windows 11, MSO'24, Dark Shadow Gray, 2.65KG, [G15-5530], Backlit Keyboard, Gaming Laptop</t>
         </is>
       </c>
       <c r="C154" t="inlineStr"/>
       <c r="D154" t="n">
-        <v>79590</v>
+        <v>89990</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="C155" t="inlineStr"/>
       <c r="D155" t="n">
-        <v>79990</v>
+        <v>79590</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>EBook 11.6" HD Laptop |</t>
+          <t>Dell G15, 13th Gen Intel</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>EBook 11.6" HD Laptop | Best Student &amp; Office Work Laptop | Celeron N4020 | 4GB DDR4 | 128GB eMMC + M.2 SSD Expandable Slot | Win 11 Home |31Wh Battery | UHD Graphics 600 | Black</t>
+          <t>Dell G15, 13th Gen Intel Core i5-13450HX Processor, NVIDIA RTX 3050-6GB, (16GB RAM 1TB SSD) FHD 15.6"/39.62 cm, Orange Backlit Keyboard, Win 11, MS Office'24, Dark Shadow Grey, 2.65Kg Gaming Laptop</t>
         </is>
       </c>
       <c r="C156" t="inlineStr"/>
       <c r="D156" t="n">
-        <v>11990</v>
+        <v>79990</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3715,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3736,7 @@
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3757,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3778,7 @@
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3799,7 @@
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -3820,7 +3820,7 @@
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -3841,7 +3841,7 @@
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -3862,7 +3862,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -3883,7 +3883,7 @@
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -3900,11 +3900,11 @@
       </c>
       <c r="C166" t="inlineStr"/>
       <c r="D166" t="n">
-        <v>16990</v>
+        <v>11990</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -3925,14 +3925,14 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ebook_11.6"_hd_laptop_|</t>
+          <t>EBook 11.6" HD Laptop |</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -3942,28 +3942,28 @@
       </c>
       <c r="C168" t="inlineStr"/>
       <c r="D168" t="n">
-        <v>10603</v>
+        <v>16990</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>hp_14_smartchoice,_intel_core</t>
+          <t>ebook_11.6"_hd_laptop_|</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>HP 14 Smartchoice, Intel Core Ultra 5 125H 12 TOPS, 24GB DDR5 (Upgradeable) 1TB SSD, Anti-Glare, FHD, 14''/35.6cm,Win11, M365*Office24, Silver, 1.4kg, ep1180tu, FHD Camera w/Shutter, Backlit AI Laptop</t>
+          <t>EBook 11.6" HD Laptop | Best Student &amp; Office Work Laptop | Celeron N4020 | 4GB DDR4 | 128GB eMMC + M.2 SSD Expandable Slot | Win 11 Home |31Wh Battery | UHD Graphics 600 | Black</t>
         </is>
       </c>
       <c r="C169" t="inlineStr"/>
       <c r="D169" t="n">
-        <v>77990</v>
+        <v>10603</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
@@ -3974,17 +3974,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>hp_14,_amd_ryzen_7</t>
+          <t>hp_14_smartchoice,_intel_core</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>HP 14, AMD Ryzen 7 7730U (16GB DDR4, 512GB SSD) FHD, Anti-Glare, Micro-Edge, 14''/35.6cm, Win11, M365 Basic(1yr), Office Home24, Silver,1.4kg, EM0104AU, FHD Camera w/Privacy Shutter, Backlit Laptop</t>
+          <t>HP 14 Smartchoice, Intel Core Ultra 5 125H 12 TOPS, 24GB DDR5 (Upgradeable) 1TB SSD, Anti-Glare, FHD, 14''/35.6cm,Win11, M365*Office24, Silver, 1.4kg, ep1180tu, FHD Camera w/Shutter, Backlit AI Laptop</t>
         </is>
       </c>
       <c r="C170" t="inlineStr"/>
       <c r="D170" t="n">
-        <v>59990</v>
+        <v>77990</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
@@ -3995,42 +3995,42 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>HP 14s Intel Celeron Dual</t>
+          <t>hp_14,_amd_ryzen_7</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>HP 14s Intel Celeron Dual Core N4500 Laptop (8GB/512GB SSD/Win 11) 14.0" HD Display, MSO 24, Black, 1.46kg, DQ3149TU Thin and Light Business Laptop</t>
+          <t>HP 14, AMD Ryzen 7 7730U (16GB DDR4, 512GB SSD) FHD, Anti-Glare, Micro-Edge, 14''/35.6cm, Win11, M365 Basic(1yr), Office Home24, Silver,1.4kg, EM0104AU, FHD Camera w/Privacy Shutter, Backlit Laptop</t>
         </is>
       </c>
       <c r="C171" t="inlineStr"/>
       <c r="D171" t="n">
-        <v>40400</v>
+        <v>59990</v>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>HP 15 (2026), AMD Athlon</t>
+          <t>HP 14s Intel Celeron Dual</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>HP 15 (2026), AMD Athlon Dual Core 7120U - (8 GB DDR5/512 GB SSD/AMD Radeon 610M Graphics/DOS) Thin and Light Business Laptop/15.6" HD Display/Turbo Silver/Copilot Key/1.5kg</t>
+          <t>HP 14s Intel Celeron Dual Core N4500 Laptop (8GB/512GB SSD/Win 11) 14.0" HD Display, MSO 24, Black, 1.46kg, DQ3149TU Thin and Light Business Laptop</t>
         </is>
       </c>
       <c r="C172" t="inlineStr"/>
       <c r="D172" t="n">
-        <v>39999</v>
+        <v>40400</v>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -4042,23 +4042,23 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>HP 15 (2026), AMD Athlon Dual Core 7120U - (8 GB DDR5/512 GB SSD/AMD Radeon 610M Graphics/Windows 11 Pro) Thin and Light Business Laptop/15.6" HD Display/Turbo Silver/Copilot Key/1.5kg/MS Office</t>
+          <t>HP 15 (2026), AMD Athlon Dual Core 7120U - (8 GB DDR5/512 GB SSD/AMD Radeon 610M Graphics/DOS) Thin and Light Business Laptop/15.6" HD Display/Turbo Silver/Copilot Key/1.5kg</t>
         </is>
       </c>
       <c r="C173" t="inlineStr"/>
       <c r="D173" t="n">
-        <v>39660</v>
+        <v>39999</v>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>hp_15_(2026),_amd_athlon</t>
+          <t>HP 15 (2026), AMD Athlon</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -4068,70 +4068,70 @@
       </c>
       <c r="C174" t="inlineStr"/>
       <c r="D174" t="n">
-        <v>41999</v>
+        <v>39660</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>HP 15 (2026), AMD Ryzen</t>
+          <t>hp_15_(2026),_amd_athlon</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>HP 15 (2026), AMD Ryzen 3 Quad Core 7335U - (8 GB DDR5/512 GB SSD/AMD Radeon 660M Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" Display/Turbo Silver/Copilot Key/1.5kg/MS Office</t>
+          <t>HP 15 (2026), AMD Athlon Dual Core 7120U - (8 GB DDR5/512 GB SSD/AMD Radeon 610M Graphics/Windows 11 Pro) Thin and Light Business Laptop/15.6" HD Display/Turbo Silver/Copilot Key/1.5kg/MS Office</t>
         </is>
       </c>
       <c r="C175" t="inlineStr"/>
       <c r="D175" t="n">
-        <v>42780</v>
+        <v>41999</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>hp_15_(i5_14th_gen),</t>
+          <t>HP 15 (2026), AMD Ryzen</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>HP 15 (i5 14th Gen), Intel Core 5, 16GB RAM (Upgradeable), 512GB SSD, FHD, Anti-Glare, 15.6''/39.6cm, Win11, M365 Basic(1yr), Office24, Silver,1.59kg, fd0682tu, FHD Camera w/Shutter, Backlit Laptop</t>
+          <t>HP 15 (2026), AMD Ryzen 3 Quad Core 7335U - (8 GB DDR5/512 GB SSD/AMD Radeon 660M Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" Display/Turbo Silver/Copilot Key/1.5kg/MS Office</t>
         </is>
       </c>
       <c r="C176" t="inlineStr"/>
       <c r="D176" t="n">
-        <v>63990</v>
+        <v>42780</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>hp_15_laptop_|_intel</t>
+          <t>hp_15_(i5_14th_gen),</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>HP 15 Laptop | Intel Core i5-13420H,13th Gen |16GB RAM | 512GB SSD | Win 11 |M365 Basic(1yr)* Office24|Anti-Glare, Micro-Edge, 15.6''/39.6cm|Backlit KB|FHD Camera w/Shutter|1.65kg, Silver -FR0045TU</t>
+          <t>HP 15 (i5 14th Gen), Intel Core 5, 16GB RAM (Upgradeable), 512GB SSD, FHD, Anti-Glare, 15.6''/39.6cm, Win11, M365 Basic(1yr), Office24, Silver,1.59kg, fd0682tu, FHD Camera w/Shutter, Backlit Laptop</t>
         </is>
       </c>
       <c r="C177" t="inlineStr"/>
       <c r="D177" t="n">
-        <v>68990</v>
+        <v>63990</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -4142,17 +4142,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>hp_15_laptop,_(14th_gen</t>
+          <t>hp_15_laptop_|_intel</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>HP 15 Laptop, (14th Gen Core i5) Intel Core 5-120U (24GB RAM, 512GB SSD, Win 11, M365 Basic(1yr)* Office24,15.6''/39.6cm FHD Anti-Glare Display, Backlit KB, FHD Camera, Dual Speakers, Silver, 1.59kg)</t>
+          <t>HP 15 Laptop | Intel Core i5-13420H,13th Gen |16GB RAM | 512GB SSD | Win 11 |M365 Basic(1yr)* Office24|Anti-Glare, Micro-Edge, 15.6''/39.6cm|Backlit KB|FHD Camera w/Shutter|1.65kg, Silver -FR0045TU</t>
         </is>
       </c>
       <c r="C178" t="inlineStr"/>
       <c r="D178" t="n">
-        <v>72800</v>
+        <v>68990</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
@@ -4163,42 +4163,42 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HP 15 Laptop, Intel (14th</t>
+          <t>hp_15_laptop,_(14th_gen</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>HP 15 Laptop, Intel (14th Gen) Core 5 120U (24GB DDR5, 512GB SSD), Micro-Edge, Anti-Glare, 15.6''/39.6cm, Win11, M365* Office24, Silver, 1.59kg, fd0262TU, FHD Camera, Backlit, Dual Speakers</t>
+          <t>HP 15 Laptop, (14th Gen Core i5) Intel Core 5-120U (24GB RAM, 512GB SSD, Win 11, M365 Basic(1yr)* Office24,15.6''/39.6cm FHD Anti-Glare Display, Backlit KB, FHD Camera, Dual Speakers, Silver, 1.59kg)</t>
         </is>
       </c>
       <c r="C179" t="inlineStr"/>
       <c r="D179" t="n">
-        <v>67990</v>
+        <v>72800</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>HP 15 Smartchoice, 13th Gen</t>
+          <t>HP 15 Laptop, Intel (14th</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>HP 15 Smartchoice, 13th Gen Intel Core i3-1315U (12GB DDR4, 512GB SSD) FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365(1yr)*Office24, Silver, 1.59kg, fd0573TU, FHD Camera w/Shutter Laptop</t>
+          <t>HP 15 Laptop, Intel (14th Gen) Core 5 120U (24GB DDR5, 512GB SSD), Micro-Edge, Anti-Glare, 15.6''/39.6cm, Win11, M365* Office24, Silver, 1.59kg, fd0262TU, FHD Camera, Backlit, Dual Speakers</t>
         </is>
       </c>
       <c r="C180" t="inlineStr"/>
       <c r="D180" t="n">
-        <v>55990</v>
+        <v>67990</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4210,16 +4210,16 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>HP 15 Smartchoice, 13th Gen Intel Core i3-1315U(8GB DDR4,512GB SSD) FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365(1yr)*Office24, Silver,1.59kg, fd0572TU, FHD Camera w/Shutter, Backlit Laptop</t>
+          <t>HP 15 Smartchoice, 13th Gen Intel Core i3-1315U (12GB DDR4, 512GB SSD) FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365(1yr)*Office24, Silver, 1.59kg, fd0573TU, FHD Camera w/Shutter Laptop</t>
         </is>
       </c>
       <c r="C181" t="inlineStr"/>
       <c r="D181" t="n">
-        <v>51990</v>
+        <v>55990</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
@@ -4261,7 +4261,7 @@
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -4303,14 +4303,14 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>hp_15_smartchoice,_13th_gen</t>
+          <t>HP 15 Smartchoice, 13th Gen</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -4320,28 +4320,28 @@
       </c>
       <c r="C186" t="inlineStr"/>
       <c r="D186" t="n">
-        <v>49990</v>
+        <v>51990</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>hp_15_smartchoice,_intel_core</t>
+          <t>hp_15_smartchoice,_13th_gen</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>HP 15 Smartchoice, Intel Core Ultra 5 125H, 12 Tops (16GB DDR5, 512GB SSD) FHD, IPS, 15.6''/39.6cm, Win11, M365(1yr)* Office24, Silver, 1.65kg, fd1254TU, FHD Camera w/Shutter, AI Powered Laptop</t>
+          <t>HP 15 Smartchoice, 13th Gen Intel Core i3-1315U(8GB DDR4,512GB SSD) FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365(1yr)*Office24, Silver,1.59kg, fd0572TU, FHD Camera w/Shutter, Backlit Laptop</t>
         </is>
       </c>
       <c r="C187" t="inlineStr"/>
       <c r="D187" t="n">
-        <v>69990</v>
+        <v>49990</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -4352,21 +4352,21 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>HP 15, 13th Gen Intel</t>
+          <t>hp_15_smartchoice,_intel_core</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>HP 15, 13th Gen Intel Core i3-1315U (8GB DDR4, 512GB SSD), FHD, Micro -Edge, Anti-Glare, 15.6''/39.6cm, Win11, M365* Office24, Silver, 1.59kg, fd0624tu, FHD Camera, UHD Graphics Laptop</t>
+          <t>HP 15 Smartchoice, Intel Core Ultra 5 125H, 12 Tops (16GB DDR5, 512GB SSD) FHD, IPS, 15.6''/39.6cm, Win11, M365(1yr)* Office24, Silver, 1.65kg, fd1254TU, FHD Camera w/Shutter, AI Powered Laptop</t>
         </is>
       </c>
       <c r="C188" t="inlineStr"/>
       <c r="D188" t="n">
-        <v>47490</v>
+        <v>69990</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -4378,16 +4378,16 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>HP 15, 13th Gen Intel Core i3-1315U Laptop (8GB DDR4,512GB SSD) Anti-Glare, Micro-Edge,15.6''/39.6cm, FHD, Win11,M365 Basic(1yr),Office Home24, Silver,1.59kg, FHD Camera w/Privacy Shutter, fd0569TU</t>
+          <t>HP 15, 13th Gen Intel Core i3-1315U (8GB DDR4, 512GB SSD), FHD, Micro -Edge, Anti-Glare, 15.6''/39.6cm, Win11, M365* Office24, Silver, 1.59kg, fd0624tu, FHD Camera, UHD Graphics Laptop</t>
         </is>
       </c>
       <c r="C189" t="inlineStr"/>
       <c r="D189" t="n">
-        <v>47990</v>
+        <v>47490</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -4408,7 +4408,7 @@
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
@@ -4425,11 +4425,11 @@
       </c>
       <c r="C191" t="inlineStr"/>
       <c r="D191" t="n">
-        <v>46990</v>
+        <v>47990</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
@@ -4450,7 +4450,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4471,7 +4471,7 @@
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
@@ -4492,7 +4492,7 @@
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -4513,7 +4513,7 @@
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
@@ -4551,11 +4551,11 @@
       </c>
       <c r="C197" t="inlineStr"/>
       <c r="D197" t="n">
-        <v>48900</v>
+        <v>46990</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-17</t>
         </is>
       </c>
     </row>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
@@ -4593,11 +4593,11 @@
       </c>
       <c r="C199" t="inlineStr"/>
       <c r="D199" t="n">
-        <v>50000</v>
+        <v>48900</v>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -4614,11 +4614,11 @@
       </c>
       <c r="C200" t="inlineStr"/>
       <c r="D200" t="n">
-        <v>49850</v>
+        <v>50000</v>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -4635,11 +4635,11 @@
       </c>
       <c r="C201" t="inlineStr"/>
       <c r="D201" t="n">
-        <v>49990</v>
+        <v>49850</v>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
@@ -4656,11 +4656,11 @@
       </c>
       <c r="C202" t="inlineStr"/>
       <c r="D202" t="n">
-        <v>49820</v>
+        <v>49990</v>
       </c>
       <c r="E202" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
@@ -4681,7 +4681,7 @@
       </c>
       <c r="E203" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -4698,11 +4698,11 @@
       </c>
       <c r="C204" t="inlineStr"/>
       <c r="D204" t="n">
-        <v>50400</v>
+        <v>49820</v>
       </c>
       <c r="E204" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -4719,11 +4719,11 @@
       </c>
       <c r="C205" t="inlineStr"/>
       <c r="D205" t="n">
-        <v>50390</v>
+        <v>50400</v>
       </c>
       <c r="E205" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -4740,11 +4740,11 @@
       </c>
       <c r="C206" t="inlineStr"/>
       <c r="D206" t="n">
-        <v>50150</v>
+        <v>50390</v>
       </c>
       <c r="E206" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -4761,11 +4761,11 @@
       </c>
       <c r="C207" t="inlineStr"/>
       <c r="D207" t="n">
-        <v>50040</v>
+        <v>50150</v>
       </c>
       <c r="E207" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="E208" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -4803,11 +4803,11 @@
       </c>
       <c r="C209" t="inlineStr"/>
       <c r="D209" t="n">
-        <v>49670</v>
+        <v>50040</v>
       </c>
       <c r="E209" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -4824,11 +4824,11 @@
       </c>
       <c r="C210" t="inlineStr"/>
       <c r="D210" t="n">
-        <v>49480</v>
+        <v>49670</v>
       </c>
       <c r="E210" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
@@ -4845,11 +4845,11 @@
       </c>
       <c r="C211" t="inlineStr"/>
       <c r="D211" t="n">
-        <v>49470</v>
+        <v>49480</v>
       </c>
       <c r="E211" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
@@ -4866,11 +4866,11 @@
       </c>
       <c r="C212" t="inlineStr"/>
       <c r="D212" t="n">
-        <v>49300</v>
+        <v>49470</v>
       </c>
       <c r="E212" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
@@ -4882,37 +4882,37 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>HP 15, 13th Gen Intel Core i3-1315U, (8GB DDR4,512GB SSD) Anti-Glare, Micro-Edge, FHD,15.6''/39.6cm, Win11,M365 Basic(1yr),Office24, Silver,1.59kg, fd0572TU, FHD Camera w/Shutter, Backlit Laptop</t>
+          <t>HP 15, 13th Gen Intel Core i3-1315U Laptop (8GB DDR4,512GB SSD) Anti-Glare, Micro-Edge,15.6''/39.6cm, FHD, Win11,M365 Basic(1yr),Office Home24, Silver,1.59kg, FHD Camera w/Privacy Shutter, fd0569TU</t>
         </is>
       </c>
       <c r="C213" t="inlineStr"/>
       <c r="D213" t="n">
-        <v>47990</v>
+        <v>49300</v>
       </c>
       <c r="E213" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>HP 15, AMD Ryzen 5</t>
+          <t>HP 15, 13th Gen Intel</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>HP 15, AMD Ryzen 5 7520U,(16GB LPDDR5, 512GB SSD), Anti-Glare, Micro-Edge, FHD, 15.6''/39.6cm, Win 11, Office 24,M365 Basic(1yr)*,Silver, 1.59kg, fc0690au, FHD Camera, Backlit KB Laptop</t>
+          <t>HP 15, 13th Gen Intel Core i3-1315U, (8GB DDR4,512GB SSD) Anti-Glare, Micro-Edge, FHD,15.6''/39.6cm, Win11,M365 Basic(1yr),Office24, Silver,1.59kg, fd0572TU, FHD Camera w/Shutter, Backlit Laptop</t>
         </is>
       </c>
       <c r="C214" t="inlineStr"/>
       <c r="D214" t="n">
-        <v>53990</v>
+        <v>47990</v>
       </c>
       <c r="E214" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
@@ -4933,7 +4933,7 @@
       </c>
       <c r="E215" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -4950,18 +4950,18 @@
       </c>
       <c r="C216" t="inlineStr"/>
       <c r="D216" t="n">
-        <v>54990</v>
+        <v>53990</v>
       </c>
       <c r="E216" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>hp_15,_amd_ryzen_5</t>
+          <t>HP 15, AMD Ryzen 5</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -4971,116 +4971,116 @@
       </c>
       <c r="C217" t="inlineStr"/>
       <c r="D217" t="n">
-        <v>61250</v>
+        <v>54990</v>
       </c>
       <c r="E217" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>HP 15, AMD Ryzen 7</t>
+          <t>hp_15,_amd_ryzen_5</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>HP 15, AMD Ryzen 7 7735HS (16GB DDR5,512GB SSD) FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365 Basic(1yr)* Office24, Silver, 1.59kg, fc1038AU, AMD Radeon FHD Camera w/Shutter, Backlit Laptop</t>
+          <t>HP 15, AMD Ryzen 5 7520U,(16GB LPDDR5, 512GB SSD), Anti-Glare, Micro-Edge, FHD, 15.6''/39.6cm, Win 11, Office 24,M365 Basic(1yr)*,Silver, 1.59kg, fc0690au, FHD Camera, Backlit KB Laptop</t>
         </is>
       </c>
       <c r="C218" t="inlineStr"/>
       <c r="D218" t="n">
-        <v>59990</v>
+        <v>61250</v>
       </c>
       <c r="E218" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>HP 15, Intel Core 5</t>
+          <t>HP 15, AMD Ryzen 7</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>HP 15, Intel Core 5 120U (14th Gen) 16GB DDR4, 512GB SSD, FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365 Basic(1yr), Office24, Silver,1.59kg, FD0640TU/682tu, FHD Camera w/Shutter, BL Laptop</t>
+          <t>HP 15, AMD Ryzen 7 7735HS (16GB DDR5,512GB SSD) FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365 Basic(1yr)* Office24, Silver, 1.59kg, fc1038AU, AMD Radeon FHD Camera w/Shutter, Backlit Laptop</t>
         </is>
       </c>
       <c r="C219" t="inlineStr"/>
       <c r="D219" t="n">
-        <v>65990</v>
+        <v>59990</v>
       </c>
       <c r="E219" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>HP 15, Intel Core Ultra</t>
+          <t>HP 15, Intel Core 5</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>HP 15, Intel Core Ultra 5 125H (24GB DDR5, 1TB SSD), Micro-Edge, Anti-Glare, FHD, 15''/39.6cm, Win11, M365* Office24, Silver, 1.65kg, FD1458TU, FHD Camera, Backlit Laptop</t>
+          <t>HP 15, Intel Core 5 120U (14th Gen) 16GB DDR4, 512GB SSD, FHD, Anti-Glare, Micro-Edge, 15.6''/39.6cm, Win11, M365 Basic(1yr), Office24, Silver,1.59kg, FD0640TU/682tu, FHD Camera w/Shutter, BL Laptop</t>
         </is>
       </c>
       <c r="C220" t="inlineStr"/>
       <c r="D220" t="n">
-        <v>84990</v>
+        <v>65990</v>
       </c>
       <c r="E220" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>hp_15,_intel_core_i3-1315u-13th</t>
+          <t>HP 15, Intel Core Ultra</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>HP 15, Intel Core i3-1315U-13th Gen Laptop (8GB DDR4 Ram,512GB SSD) Anti-Glare, Micro-Edge,15.6'" FHD, Win11,M365 Basic(1yr),Office Home24, Silver,1.59kg, FHD Camera Shutter, 15-fd0569TU</t>
+          <t>HP 15, Intel Core Ultra 5 125H (24GB DDR5, 1TB SSD), Micro-Edge, Anti-Glare, FHD, 15''/39.6cm, Win11, M365* Office24, Silver, 1.65kg, FD1458TU, FHD Camera, Backlit Laptop</t>
         </is>
       </c>
       <c r="C221" t="inlineStr"/>
       <c r="D221" t="n">
-        <v>49490</v>
+        <v>84990</v>
       </c>
       <c r="E221" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>HP 255R G10 Notebook (AMD</t>
+          <t>hp_15,_intel_core_i3-1315u-13th</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>HP 255R G10 Notebook (AMD Athlon Silver 7120U /8GB/512GB/DOS) 15.6-inch(39.6cm), Anti-Glare, HD Laptop, Radeon Graphics, Silver,1.52kg</t>
+          <t>HP 15, Intel Core i3-1315U-13th Gen Laptop (8GB DDR4 Ram,512GB SSD) Anti-Glare, Micro-Edge,15.6'" FHD, Win11,M365 Basic(1yr),Office Home24, Silver,1.59kg, FHD Camera Shutter, 15-fd0569TU</t>
         </is>
       </c>
       <c r="C222" t="inlineStr"/>
       <c r="D222" t="n">
-        <v>41700</v>
+        <v>49490</v>
       </c>
       <c r="E222" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -5097,11 +5097,11 @@
       </c>
       <c r="C223" t="inlineStr"/>
       <c r="D223" t="n">
-        <v>39340</v>
+        <v>41700</v>
       </c>
       <c r="E223" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -5118,11 +5118,11 @@
       </c>
       <c r="C224" t="inlineStr"/>
       <c r="D224" t="n">
-        <v>40409</v>
+        <v>39340</v>
       </c>
       <c r="E224" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -5139,11 +5139,11 @@
       </c>
       <c r="C225" t="inlineStr"/>
       <c r="D225" t="n">
-        <v>39618</v>
+        <v>40409</v>
       </c>
       <c r="E225" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
@@ -5160,65 +5160,65 @@
       </c>
       <c r="C226" t="inlineStr"/>
       <c r="D226" t="n">
-        <v>39525</v>
+        <v>39618</v>
       </c>
       <c r="E226" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>HP Omen, Intel Core Ultra</t>
+          <t>HP 255R G10 Notebook (AMD</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>HP Omen, Intel Core Ultra 7 255H, 8GB RTX 5050, 24GB DDR5(Upgradeable) 1TB SSD, 2K, 165Hz, 3ms Response time, IPS, 16''/40.6cm, Win11, M365*Office24, Shadow Black, 2.43kg, am0240tx, RGB Gaming Laptop</t>
+          <t>HP 255R G10 Notebook (AMD Athlon Silver 7120U /8GB/512GB/DOS) 15.6-inch(39.6cm), Anti-Glare, HD Laptop, Radeon Graphics, Silver,1.52kg</t>
         </is>
       </c>
       <c r="C227" t="inlineStr"/>
       <c r="D227" t="n">
-        <v>129990</v>
+        <v>39525</v>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>HP OmniBook 3, AMD Ryzen</t>
+          <t>HP Omen, Intel Core Ultra</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>HP OmniBook 3, AMD Ryzen AI 5 330 (24GB DDR5 RAM, 1TB SSD) FHD, Anti-Glare, 15.6''/39.6cm, Win11, Office24, Glacier Silver,1.7kg, fn0074AU, FHD Camera w/Shutter, FPR, Backlit KB, Next Gen AI Laptop</t>
+          <t>HP Omen, Intel Core Ultra 7 255H, 8GB RTX 5050, 24GB DDR5(Upgradeable) 1TB SSD, 2K, 165Hz, 3ms Response time, IPS, 16''/40.6cm, Win11, M365*Office24, Shadow Black, 2.43kg, am0240tx, RGB Gaming Laptop</t>
         </is>
       </c>
       <c r="C228" t="inlineStr"/>
       <c r="D228" t="n">
-        <v>69990</v>
+        <v>129990</v>
       </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>HP OmniBook 5 OLED (Previously</t>
+          <t>HP OmniBook 3, AMD Ryzen</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>HP OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 1TB SSD) 2K, 14''/35.6cm, Win11, M365 Basic(1yr)* Office24, Silver, 1.35kg, he0015QU, Light-Weight, Next-Gen AI Laptop</t>
+          <t>HP OmniBook 3, AMD Ryzen AI 5 330 (24GB DDR5 RAM, 1TB SSD) FHD, Anti-Glare, 15.6''/39.6cm, Win11, Office24, Glacier Silver,1.7kg, fn0074AU, FHD Camera w/Shutter, FPR, Backlit KB, Next Gen AI Laptop</t>
         </is>
       </c>
       <c r="C229" t="inlineStr"/>
@@ -5227,7 +5227,7 @@
       </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
@@ -5239,16 +5239,16 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>HP OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 512GB SSD) 2K, 14''/35.6cm, Win11, M365 Basic(1yr)* Office24, Silver, 1.35kg, he0014QU, Light-Weight, Next-Gen AI Laptop</t>
+          <t>HP OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 1TB SSD) 2K, 14''/35.6cm, Win11, M365 Basic(1yr)* Office24, Silver, 1.35kg, he0015QU, Light-Weight, Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C230" t="inlineStr"/>
       <c r="D230" t="n">
-        <v>78990</v>
+        <v>69990</v>
       </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
@@ -5265,154 +5265,154 @@
       </c>
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="n">
-        <v>66990</v>
+        <v>78990</v>
       </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>hp_omnibook_3,_snapdragon_x</t>
+          <t>HP OmniBook 5 OLED (Previously</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>HP Omnibook 3, Snapdragon X Processor 45 TOPS (16GB LPDDR5x,512GB SSD) 2K WUXGA, Anti-Glare, 14''/35.6cm, Win 11, M365*Office 24,Silver,1.42kg, hz0026QU, Lighter mini Charger, FHD IR Camera, AI Laptop</t>
+          <t>HP OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 512GB SSD) 2K, 14''/35.6cm, Win11, M365 Basic(1yr)* Office24, Silver, 1.35kg, he0014QU, Light-Weight, Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
       <c r="D232" t="n">
-        <v>79990</v>
+        <v>66990</v>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>HP Omnibook 3, Snapdragon X</t>
+          <t>hp_omnibook_x_flip_oled</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>HP Omnibook 3, Snapdragon X Processor, 45 TOPS (16GB LPDDR5x, 512GB SSD) 2K, WUXGA, IPS, 14''/35.6cm, Win 11, Office 24, Silver, 1.4kg, hz0026QU, FHD IR Camera, 42% Lighter mini GaN Charger, AI Laptop</t>
+          <t>HP OmniBook X Flip OLED Intel Core Ultra 5 226V, 40 Tops (16GB LPDDR5x,1TB SSD) 3K, Touch, 120hz, 14''/35.6cm, Intel ARC Graphic,Win11, Office24, Meteor Silver, 1.38kg, fm0099TU,Pen, 2 in 1 AI Laptop</t>
         </is>
       </c>
       <c r="C233" t="inlineStr"/>
       <c r="D233" t="n">
-        <v>69990</v>
+        <v>115990</v>
       </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>HP Omnibook 3, Snapdragon X</t>
+          <t>hp_omnibook_3,_snapdragon_x</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>HP Omnibook 3, Snapdragon X Processor, 45 TOPS (16GB LPDDR5x, 512GB SSD) 2K, WUXGA, IPS, 14''/35.6cm, Win 11, Office 24, Silver, 1.4kg, hz0026QU, FHD IR Camera, 42% Lighter mini GaN Charger, AI Laptop</t>
+          <t>HP Omnibook 3, Snapdragon X Processor 45 TOPS (16GB LPDDR5x,512GB SSD) 2K WUXGA, Anti-Glare, 14''/35.6cm, Win 11, M365*Office 24,Silver,1.42kg, hz0026QU, Lighter mini Charger, FHD IR Camera, AI Laptop</t>
         </is>
       </c>
       <c r="C234" t="inlineStr"/>
       <c r="D234" t="n">
-        <v>73990</v>
+        <v>79990</v>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>HP Omnibook 5 OLED (Previously</t>
+          <t>HP Omnibook 3, Snapdragon X</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>HP Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x,1TB SSD) 2K OLED,16''/40.6cm, Win11, M365*Office24, Glacier Silver, 1.59kg, fb0001QU, Backlit, Next-Gen AI Laptop</t>
+          <t>HP Omnibook 3, Snapdragon X Processor, 45 TOPS (16GB LPDDR5x, 512GB SSD) 2K, WUXGA, IPS, 14''/35.6cm, Win 11, Office 24, Silver, 1.4kg, hz0026QU, FHD IR Camera, 42% Lighter mini GaN Charger, AI Laptop</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
       <c r="D235" t="n">
-        <v>78850</v>
+        <v>69990</v>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>hp_omnibook_5_oled_(previously</t>
+          <t>HP Omnibook 3, Snapdragon X</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>HP Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor 45 Tops (16GB LPDDR5x, 1TB SSD) 2K,16''/40.6cm, Win11, Office24, Silver, 1.59kg, fb0001QU, Multi-Day Battery AI Laptop</t>
+          <t>HP Omnibook 3, Snapdragon X Processor, 45 TOPS (16GB LPDDR5x, 512GB SSD) 2K, WUXGA, IPS, 14''/35.6cm, Win 11, Office 24, Silver, 1.4kg, hz0026QU, FHD IR Camera, 42% Lighter mini GaN Charger, AI Laptop</t>
         </is>
       </c>
       <c r="C236" t="inlineStr"/>
       <c r="D236" t="n">
-        <v>77900</v>
+        <v>73990</v>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>hp_pavilion_plus,_intel_core</t>
+          <t>HP Omnibook 5 OLED (Previously</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>HP Pavilion Plus, Intel Core i5-1335U-13th Gen Laptop, (16GB LPDDR5x,512GB SSD),IPS, 300 nits, 14''(35.6cm) 2K,Win 11, M365 Basic(1yr), Office Home 24, Silver,1.38kg, 5MP Camera w/Shutter, ew0107TU</t>
+          <t>HP Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x,1TB SSD) 2K OLED,16''/40.6cm, Win11, M365*Office24, Glacier Silver, 1.59kg, fb0001QU, Backlit, Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C237" t="inlineStr"/>
       <c r="D237" t="n">
-        <v>63990</v>
+        <v>78850</v>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>hp_professional_15_(2026),_intel</t>
+          <t>hp_omnibook_5_oled_(previously</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>HP Professional 15 (2026), Intel (i3 14th Gen) Core 3 100U - (8 GB/512 GB SSD/Intel UHD Graphics/Windows 11 Home) Thin &amp; Light Business Laptop/15.6" Display/Turbo Silver/Copilot Key/1.5kg/MS Office</t>
+          <t>HP Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor 45 Tops (16GB LPDDR5x, 1TB SSD) 2K,16''/40.6cm, Win11, Office24, Silver, 1.59kg, fb0001QU, Multi-Day Battery AI Laptop</t>
         </is>
       </c>
       <c r="C238" t="inlineStr"/>
       <c r="D238" t="n">
-        <v>48990</v>
+        <v>77900</v>
       </c>
       <c r="E238" t="inlineStr">
         <is>
@@ -5423,42 +5423,42 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>HP Smartchoice OmniBook 5 OLED</t>
+          <t>hp_pavilion_plus,_intel_core</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 1TB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)*Office24, Silver,1.35kg, he0015QU,Light-Weight,Next-Gen AI Laptop</t>
+          <t>HP Pavilion Plus, Intel Core i5-1335U-13th Gen Laptop, (16GB LPDDR5x,512GB SSD),IPS, 300 nits, 14''(35.6cm) 2K,Win 11, M365 Basic(1yr), Office Home 24, Silver,1.38kg, 5MP Camera w/Shutter, ew0107TU</t>
         </is>
       </c>
       <c r="C239" t="inlineStr"/>
       <c r="D239" t="n">
-        <v>82990</v>
+        <v>63990</v>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>HP Smartchoice OmniBook 5 OLED</t>
+          <t>hp_professional_15_(2026),_intel</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 1TB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)*Office24, Silver,1.35kg, he0015QU,Light-Weight,Next-Gen AI Laptop</t>
+          <t>HP Professional 15 (2026), Intel (i3 14th Gen) Core 3 100U - (8 GB/512 GB SSD/Intel UHD Graphics/Windows 11 Home) Thin &amp; Light Business Laptop/15.6" Display/Turbo Silver/Copilot Key/1.5kg/MS Office</t>
         </is>
       </c>
       <c r="C240" t="inlineStr"/>
       <c r="D240" t="n">
-        <v>76990</v>
+        <v>48990</v>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -5470,16 +5470,16 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 512GB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)* Office24, Silver, 1.35kg, he0014QU, Next-Gen AI Laptop</t>
+          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 1TB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)*Office24, Silver,1.35kg, he0015QU,Light-Weight,Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C241" t="inlineStr"/>
       <c r="D241" t="n">
-        <v>78990</v>
+        <v>82990</v>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -5491,58 +5491,58 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 512GB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)* Office24, Silver, 1.35kg, he0014QU, Next-Gen AI Laptop</t>
+          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 1TB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)*Office24, Silver,1.35kg, he0015QU,Light-Weight,Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
       <c r="D242" t="n">
-        <v>79990</v>
+        <v>76990</v>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>HP Smartchoice Omnibook 5 OLED</t>
+          <t>HP Smartchoice OmniBook 5 OLED</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>HP Smartchoice Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x,1TB SSD) 2K OLED,16''/40.6cm, Win11, M365(1yr)*Office24, Glacier Silver, 1.59kg, fb0001QU,Next-Gen AI Laptop</t>
+          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 512GB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)* Office24, Silver, 1.35kg, he0014QU, Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C243" t="inlineStr"/>
       <c r="D243" t="n">
-        <v>68739</v>
+        <v>78990</v>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>HP Smartchoice Omnibook 5 OLED</t>
+          <t>HP Smartchoice OmniBook 5 OLED</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>HP Smartchoice Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x,1TB SSD) 2K OLED,16''/40.6cm, Win11, M365(1yr)*Office24, Glacier Silver, 1.59kg, fb0001QU,Next-Gen AI Laptop</t>
+          <t>HP Smartchoice OmniBook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x, 512GB SSD) 2K, 14''/35.6cm, Win11, M365(1yr)* Office24, Silver, 1.35kg, he0014QU, Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C244" t="inlineStr"/>
       <c r="D244" t="n">
-        <v>68739</v>
+        <v>79990</v>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -5563,7 +5563,7 @@
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
@@ -5580,11 +5580,11 @@
       </c>
       <c r="C246" t="inlineStr"/>
       <c r="D246" t="n">
-        <v>68323</v>
+        <v>68739</v>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -5601,11 +5601,11 @@
       </c>
       <c r="C247" t="inlineStr"/>
       <c r="D247" t="n">
-        <v>67940</v>
+        <v>68739</v>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
@@ -5622,74 +5622,74 @@
       </c>
       <c r="C248" t="inlineStr"/>
       <c r="D248" t="n">
-        <v>67940</v>
+        <v>68323</v>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>HP Smartchoice Victus, 13th Gen</t>
+          <t>HP Smartchoice Omnibook 5 OLED</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>HP Smartchoice Victus, 13th Gen Intel Core i7-13620H, 8GB RTX 5050, 24GB DDR5(Upgradeable) 1TB SSD, 144Hz, FHD, 15.6''/39.6cm, Win11, M365* Office24, Mica Silver, 2.29kg, fa2309TX, RGB Gaming Laptop</t>
+          <t>HP Smartchoice Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x,1TB SSD) 2K OLED,16''/40.6cm, Win11, M365(1yr)*Office24, Glacier Silver, 1.59kg, fb0001QU,Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C249" t="inlineStr"/>
       <c r="D249" t="n">
-        <v>112990</v>
+        <v>67940</v>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>HP Smartchoice Victus, AMD Ryzen</t>
+          <t>HP Smartchoice Omnibook 5 OLED</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>HP Smartchoice Victus, AMD Ryzen 7 7445HS, 6GB RTX 3050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, 15.6''/39.6cm, Win 11, M365* Office24, Blue, 2.29kg, fb3134AX/3120ax, Gaming Laptop</t>
+          <t>HP Smartchoice Omnibook 5 OLED (Previously Pavilion), Snapdragon X Processor (16GB LPDDR5x,1TB SSD) 2K OLED,16''/40.6cm, Win11, M365(1yr)*Office24, Glacier Silver, 1.59kg, fb0001QU,Next-Gen AI Laptop</t>
         </is>
       </c>
       <c r="C250" t="inlineStr"/>
       <c r="D250" t="n">
-        <v>78990</v>
+        <v>67940</v>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>HP Smartchoice Victus, AMD Ryzen</t>
+          <t>HP Smartchoice Victus, 13th Gen</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>HP Smartchoice Victus, AMD Ryzen 7 7445HS, 6GB RTX 3050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, 15.6''/39.6cm, Win 11, M365* Office24, Blue, 2.29kg, fb3134AX/3120ax, Gaming Laptop</t>
+          <t>HP Smartchoice Victus, 13th Gen Intel Core i7-13620H, 8GB RTX 5050, 24GB DDR5(Upgradeable) 1TB SSD, 144Hz, FHD, 15.6''/39.6cm, Win11, M365* Office24, Mica Silver, 2.29kg, fa2309TX, RGB Gaming Laptop</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
       <c r="D251" t="n">
-        <v>86990</v>
+        <v>112990</v>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -5706,74 +5706,74 @@
       </c>
       <c r="C252" t="inlineStr"/>
       <c r="D252" t="n">
-        <v>86990</v>
+        <v>78990</v>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>HP Victus, 14th Gen Intel</t>
+          <t>HP Smartchoice Victus, AMD Ryzen</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>HP Victus, 14th Gen Intel Core i5-14450HX, 6GB RTX 3050, 24GB DDR5, 512GB SSD, FHD, 144Hz, 300 nits, IPS,15.6''/39.6cm, Win11, M365* Office24, Mica Silver, 2.3kg, fa2303tx/fa2315tx, RGB Gaming Laptop</t>
+          <t>HP Smartchoice Victus, AMD Ryzen 7 7445HS, 6GB RTX 3050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, 15.6''/39.6cm, Win 11, M365* Office24, Blue, 2.29kg, fb3134AX/3120ax, Gaming Laptop</t>
         </is>
       </c>
       <c r="C253" t="inlineStr"/>
       <c r="D253" t="n">
-        <v>103990</v>
+        <v>86990</v>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>HP Victus, AMD Ryzen 7</t>
+          <t>HP Smartchoice Victus, AMD Ryzen</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>HP Victus, AMD Ryzen 7 7445HS, 4GB RTX 2050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, IPS, 15.6'', Win11, M365* Office24, Blue, 2.29kg, fb3189ax /3122/ 23ax Backlit, Gaming Laptop</t>
+          <t>HP Smartchoice Victus, AMD Ryzen 7 7445HS, 6GB RTX 3050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, 15.6''/39.6cm, Win 11, M365* Office24, Blue, 2.29kg, fb3134AX/3120ax, Gaming Laptop</t>
         </is>
       </c>
       <c r="C254" t="inlineStr"/>
       <c r="D254" t="n">
-        <v>65990</v>
+        <v>86990</v>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>HP Victus, AMD Ryzen 7</t>
+          <t>HP Victus, 14th Gen Intel</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>HP Victus, AMD Ryzen 7 7445HS, 4GB RTX 2050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, IPS, 15.6'', Win11, M365* Office24, Blue, 2.29kg, fb3189ax /3122/ 23ax Backlit, Gaming Laptop</t>
+          <t>HP Victus, 14th Gen Intel Core i5-14450HX, 6GB RTX 3050, 24GB DDR5, 512GB SSD, FHD, 144Hz, 300 nits, IPS,15.6''/39.6cm, Win11, M365* Office24, Mica Silver, 2.3kg, fa2303tx/fa2315tx, RGB Gaming Laptop</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
       <c r="D255" t="n">
-        <v>65990</v>
+        <v>103990</v>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
@@ -5785,16 +5785,16 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>HP Victus, AMD Ryzen 7 7445HS, 6GB RTX 4050, 16GB DDR5(Upgradeable) 512GB SSD, 144Hz, IPS, 300nits, FHD, 15.6''/39.6cm, Win11, M365* Office24, Blue, 2.29kg, fb3130AX, Backlit, DTS Audio, Gaming Laptop</t>
+          <t>HP Victus, AMD Ryzen 7 7445HS, 4GB RTX 2050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, IPS, 15.6'', Win11, M365* Office24, Blue, 2.29kg, fb3189ax /3122/ 23ax Backlit, Gaming Laptop</t>
         </is>
       </c>
       <c r="C256" t="inlineStr"/>
       <c r="D256" t="n">
-        <v>90990</v>
+        <v>65990</v>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -5806,138 +5806,138 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>HP Victus, AMD Ryzen 7 7445HS, 6GB RTX 4050, 16GB DDR5(Upgradeable) 512GB SSD, 144Hz, IPS, 300nits, FHD, 15.6''/39.6cm, Win11, M365* Office24, Blue, 2.29kg, fb3130AX, Backlit, DTS Audio, Gaming Laptop</t>
+          <t>HP Victus, AMD Ryzen 7 7445HS, 4GB RTX 2050, 16GB DDR5(Upgradeable) 512GB SSD, FHD, 144Hz, 300 nits, IPS, 15.6'', Win11, M365* Office24, Blue, 2.29kg, fb3189ax /3122/ 23ax Backlit, Gaming Laptop</t>
         </is>
       </c>
       <c r="C257" t="inlineStr"/>
       <c r="D257" t="n">
-        <v>91990</v>
+        <v>65990</v>
       </c>
       <c r="E257" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Lenovo Chromebook Intel Celeron N4500</t>
+          <t>HP Victus, AMD Ryzen 7</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Lenovo Chromebook Intel Celeron N4500 (4GB RAM/64GB eMMC 5.1/11.6 Inch (29.46cm)/HD Display/2Wx2 Stereo Speakers/HD Camera/Chrome OS/Blue/1.21Kg), 82UY0014HA</t>
+          <t>HP Victus, AMD Ryzen 7 7445HS, 6GB RTX 4050, 16GB DDR5(Upgradeable) 512GB SSD, 144Hz, IPS, 300nits, FHD, 15.6''/39.6cm, Win11, M365* Office24, Blue, 2.29kg, fb3130AX, Backlit, DTS Audio, Gaming Laptop</t>
         </is>
       </c>
       <c r="C258" t="inlineStr"/>
       <c r="D258" t="n">
-        <v>21990</v>
+        <v>90990</v>
       </c>
       <c r="E258" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Lenovo Chromebook Intel Celeron N4500</t>
+          <t>HP Victus, AMD Ryzen 7</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Lenovo Chromebook Intel Celeron N4500 (4GB RAM/64GB eMMC 5.1/11.6 Inch (29.46cm)/HD Display/2Wx2 Stereo Speakers/HD Camera/Chrome OS/Blue/1.21Kg), 82UY0014HA</t>
+          <t>HP Victus, AMD Ryzen 7 7445HS, 6GB RTX 4050, 16GB DDR5(Upgradeable) 512GB SSD, 144Hz, IPS, 300nits, FHD, 15.6''/39.6cm, Win11, M365* Office24, Blue, 2.29kg, fb3130AX, Backlit, DTS Audio, Gaming Laptop</t>
         </is>
       </c>
       <c r="C259" t="inlineStr"/>
       <c r="D259" t="n">
-        <v>18990</v>
+        <v>91990</v>
       </c>
       <c r="E259" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Lenovo IdeaPad Slim 3 13th</t>
+          <t>Lenovo Chromebook Intel Celeron N4500</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Lenovo IdeaPad Slim 3 13th Gen Intel Core i5-13420H 15.3 inch (38.8cm) WUXGA IPS Laptop (16GB RAM/1TB SSD/Windows 11/MSO 365 Basic+Office 2024/Top Metal Cover/Backlit KB/Grey/1.6Kg), 83K100S0IN</t>
+          <t>Lenovo Chromebook Intel Celeron N4500 (4GB RAM/64GB eMMC 5.1/11.6 Inch (29.46cm)/HD Display/2Wx2 Stereo Speakers/HD Camera/Chrome OS/Blue/1.21Kg), 82UY0014HA</t>
         </is>
       </c>
       <c r="C260" t="inlineStr"/>
       <c r="D260" t="n">
-        <v>70990</v>
+        <v>21990</v>
       </c>
       <c r="E260" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>lenovo_ideapad_slim_3_13th</t>
+          <t>Lenovo Chromebook Intel Celeron N4500</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Lenovo IdeaPad Slim 3 13th Gen Intel Core i7 13620H, 16GB RAM, 512GB SSD, WUXGA IPS, 15.3"/38.8cm, Win 11, Office 2024, Top Metal Cover Grey, 1.6Kg, 83K100CJIN/S1IN, Backlit KB, Laptop</t>
+          <t>Lenovo Chromebook Intel Celeron N4500 (4GB RAM/64GB eMMC 5.1/11.6 Inch (29.46cm)/HD Display/2Wx2 Stereo Speakers/HD Camera/Chrome OS/Blue/1.21Kg), 82UY0014HA</t>
         </is>
       </c>
       <c r="C261" t="inlineStr"/>
       <c r="D261" t="n">
-        <v>81990</v>
+        <v>18990</v>
       </c>
       <c r="E261" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>lenovo_ideapad_slim_3,_13th</t>
+          <t>Lenovo IdeaPad Slim 3 13th</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Lenovo IdeaPad Slim 3, 13th Gen Intel Core i5 13420H, 24GB RAM, 1TB SSD, WUXGA IPS, 15.3"/38.8cm, Windows 11, Office Home 2024, Grey, 1.6Kg, Backlit Keyboard, 1Yr ADP Free, 83K100PLIN, Laptop</t>
+          <t>Lenovo IdeaPad Slim 3 13th Gen Intel Core i5-13420H 15.3 inch (38.8cm) WUXGA IPS Laptop (16GB RAM/1TB SSD/Windows 11/MSO 365 Basic+Office 2024/Top Metal Cover/Backlit KB/Grey/1.6Kg), 83K100S0IN</t>
         </is>
       </c>
       <c r="C262" t="inlineStr"/>
       <c r="D262" t="n">
-        <v>79990</v>
+        <v>70990</v>
       </c>
       <c r="E262" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>lenovo_ideapad_slim_3,_amd</t>
+          <t>lenovo_ideapad_slim_3_13th</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Lenovo IdeaPad Slim 3, AMD Ryzen 7 8840HS, 24GB RAM, 1TB SSD, WUXGA IPS, AI PC, 15.3"/38.8cm, Backlit Keyboard, Windows 11, Office Home 2024, Grey, 1.6Kg, 1Yr ADP Free, 83KA004TIN, AI Powered Laptop</t>
+          <t>Lenovo IdeaPad Slim 3 13th Gen Intel Core i5-13420H 15.3 inch (38.8cm) WUXGA IPS Laptop (16GB RAM/512GB SSD/Windows 11/Office 2024/Top Metal Cover/Backlit KB/Luna Grey/1.6Kg), 83K101JEIN</t>
         </is>
       </c>
       <c r="C263" t="inlineStr"/>
       <c r="D263" t="n">
-        <v>87990</v>
+        <v>74990</v>
       </c>
       <c r="E263" t="inlineStr">
         <is>
@@ -5948,210 +5948,210 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Lenovo Ideapad Slim 3 AMD</t>
+          <t>lenovo_ideapad_slim_3,_13th</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Lenovo Ideapad Slim 3 AMD Ryzen 5 7520U 15.6" (39.6cm) FHD Thin and Light Laptop (16GB/512GB SSD/Windows 11/Microsoft 365 Basic + Office Home 2024/Backlit Keyboard/Grey/1.6Kg), 82XQ00XDIN</t>
+          <t>Lenovo IdeaPad Slim 3, 13th Gen Intel Core i5 13420H, 24GB RAM, 1TB SSD, WUXGA IPS, 15.3"/38.8cm, Windows 11, Office Home 2024, Grey, 1.6Kg, Backlit Keyboard, 1Yr ADP Free, 83K100PLIN, Laptop</t>
         </is>
       </c>
       <c r="C264" t="inlineStr"/>
       <c r="D264" t="n">
-        <v>50750</v>
+        <v>79990</v>
       </c>
       <c r="E264" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Lenovo LOQ 2024, Intel Core</t>
+          <t>lenovo_ideapad_slim_3,_amd</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Lenovo LOQ 2024, Intel Core i5-13450HX, 13th Gen, NVIDIA RTX 4050-6GB, 16GB RAM, 512GB SSD, FHD 144Hz, 15.6"/39.6cm, Windows 11, Office Home 2024, Grey, 2.4Kg, 83DV018JIN, 1Yr ADP Free Gaming Laptop</t>
+          <t>Lenovo IdeaPad Slim 3, AMD Ryzen 7 8840HS, 24GB RAM, 1TB SSD, WUXGA IPS, AI PC, 15.3"/38.8cm, Backlit Keyboard, Windows 11, Office Home 2024, Grey, 1.6Kg, 1Yr ADP Free, 83KA004TIN, AI Powered Laptop</t>
         </is>
       </c>
       <c r="C265" t="inlineStr"/>
       <c r="D265" t="n">
-        <v>100544</v>
+        <v>87990</v>
       </c>
       <c r="E265" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Lenovo LOQ 2025 AMD Ryzen</t>
+          <t>lenovo_ideapad_slim_5,_amd</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Lenovo LOQ 2025 AMD Ryzen 7 250| NVIDIA RTX 5050 8GB (16GB RAM/1TB SSD/144Hz Refresh Rate/440 AI TOPS/15.6" (39.6cm)/Windows 11/Office 2024/3 Mon. Game Pass/Grey/2.4Kg), 83JG008KIN</t>
+          <t>Lenovo IdeaPad Slim 5, AMD Ryzen 5 7535HS, 16GB RAM, 512GB SSD, WUXGA IPS, 13.3"/33.7cm, Windows 11, Microsoft 365 Basic + Office 2024, Grey, 1.6Kg, Backlit KB, 1Yr ADP Free, 83J2004HIN, Laptop</t>
         </is>
       </c>
       <c r="C266" t="inlineStr"/>
       <c r="D266" t="n">
-        <v>134990</v>
+        <v>72990</v>
       </c>
       <c r="E266" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Lenovo LOQ 2025 Intel Core</t>
+          <t>Lenovo Ideapad Slim 3 AMD</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Lenovo LOQ 2025 Intel Core i7-14700HX| NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/144Hz Refresh Rate/572 AI TOPS/15.6" (39.6cm)/Windows 11/Office 2024/3 Mon. Game Pass/Grey/2.4Kg), 83JE00T3IN</t>
+          <t>Lenovo Ideapad Slim 3 AMD Ryzen 5 7520U 15.6" (39.6cm) FHD Thin and Light Laptop (16GB/512GB SSD/Windows 11/Microsoft 365 Basic + Office Home 2024/Backlit Keyboard/Grey/1.6Kg), 82XQ00XDIN</t>
         </is>
       </c>
       <c r="C267" t="inlineStr"/>
       <c r="D267" t="n">
-        <v>157990</v>
+        <v>50750</v>
       </c>
       <c r="E267" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Lenovo LOQ AMD Ryzen 5</t>
+          <t>Lenovo LOQ 2024, Intel Core</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Lenovo LOQ AMD Ryzen 5 7235HS | NVIDIA RTX 4050 6GB (16GB RAM/512GB SSD/144Hz Refresh Rate/15.6" (39.6cm)/Windows 11/Office Home 2024/3 Mon. Game Pass/Grey/2.4Kg), 83JC00NYIN AI Gaming Laptop</t>
+          <t>Lenovo LOQ 2024, Intel Core i5-13450HX, 13th Gen, NVIDIA RTX 4050-6GB, 16GB RAM, 512GB SSD, FHD 144Hz, 15.6"/39.6cm, Windows 11, Office Home 2024, Grey, 2.4Kg, 83DV018JIN, 1Yr ADP Free Gaming Laptop</t>
         </is>
       </c>
       <c r="C268" t="inlineStr"/>
       <c r="D268" t="n">
-        <v>88990</v>
+        <v>100544</v>
       </c>
       <c r="E268" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Lenovo LOQ, 13th Gen Intel</t>
+          <t>Lenovo LOQ 2025 AMD Ryzen</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Lenovo LOQ, 13th Gen Intel Core i7 13700HX, RTX 5050-8GB, 16GB RAM, 1TB SSD, FHD, 15.6"/39.6cm, 144Hz, Windows 11, Office 2024, Grey, 2.4Kg, 440 AI Tops, 3 Mon. Game Pass, 83JE00U7IN, AI Gaming Laptop</t>
+          <t>Lenovo LOQ 2025 AMD Ryzen 7 250| NVIDIA RTX 5050 8GB (16GB RAM/1TB SSD/144Hz Refresh Rate/440 AI TOPS/15.6" (39.6cm)/Windows 11/Office 2024/3 Mon. Game Pass/Grey/2.4Kg), 83JG008KIN</t>
         </is>
       </c>
       <c r="C269" t="inlineStr"/>
       <c r="D269" t="n">
-        <v>121869</v>
+        <v>134990</v>
       </c>
       <c r="E269" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-05-23</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Lenovo Legion 7 2025 Intel</t>
+          <t>Lenovo LOQ 2025 Intel Core</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Lenovo Legion 7 2025 Intel Core Ultra 9 275HX| NVIDIA RTX 5070 8GB (32GB RAM/1TB SSD/WQXGA OLED/240Hz/16(40.64cm)/Windows 11/Office 2024+AI Now/White/2.0Kg), 83KY001GIN AI Powered Gaming Laptop</t>
+          <t>Lenovo LOQ 2025 Intel Core i7-14700HX| NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/144Hz Refresh Rate/572 AI TOPS/15.6" (39.6cm)/Windows 11/Office 2024/3 Mon. Game Pass/Grey/2.4Kg), 83JE00T3IN</t>
         </is>
       </c>
       <c r="C270" t="inlineStr"/>
       <c r="D270" t="n">
-        <v>239391</v>
+        <v>157990</v>
       </c>
       <c r="E270" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 5 2025</t>
+          <t>Lenovo LOQ AMD Ryzen 5</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 5 2025 AMD Ryzen 9 9955HX | NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/WQXGA OLED/165Hz/16 (40.6cm)/Windows 11/Office 2024+AI Now/Black/2.3Kg), 83F2004CIN AI Powered Gaming Laptop</t>
+          <t>Lenovo LOQ AMD Ryzen 5 7235HS | NVIDIA RTX 4050 6GB (16GB RAM/512GB SSD/144Hz Refresh Rate/15.6" (39.6cm)/Windows 11/Office Home 2024/3 Mon. Game Pass/Grey/2.4Kg), 83JC00NYIN AI Gaming Laptop</t>
         </is>
       </c>
       <c r="C271" t="inlineStr"/>
       <c r="D271" t="n">
-        <v>245490</v>
+        <v>88990</v>
       </c>
       <c r="E271" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 5 2025</t>
+          <t>Lenovo LOQ, 13th Gen Intel</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 5 2025 AMD Ryzen 9 9955HX | NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/WQXGA OLED/165Hz/16 (40.6cm)/Windows 11/Office 2024+AI Now/Black/2.3Kg), 83F2004CIN AI Powered Gaming Laptop</t>
+          <t>Lenovo LOQ, 13th Gen Intel Core i7 13700HX, RTX 5050-8GB, 16GB RAM, 1TB SSD, FHD, 15.6"/39.6cm, 144Hz, Windows 11, Office 2024, Grey, 2.4Kg, 440 AI Tops, 3 Mon. Game Pass, 83JE00U7IN, AI Gaming Laptop</t>
         </is>
       </c>
       <c r="C272" t="inlineStr"/>
       <c r="D272" t="n">
-        <v>245490</v>
+        <v>121869</v>
       </c>
       <c r="E272" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 5 2025</t>
+          <t>Lenovo Legion 7 2025 Intel</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 5 2025 AMD Ryzen 9 9955HX | NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/WQXGA OLED/165Hz/16 (40.6cm)/Windows 11/Office 2024+AI Now/Black/2.3Kg), 83F2004CIN AI Powered Gaming Laptop</t>
+          <t>Lenovo Legion 7 2025 Intel Core Ultra 9 275HX| NVIDIA RTX 5070 8GB (32GB RAM/1TB SSD/WQXGA OLED/240Hz/16(40.64cm)/Windows 11/Office 2024+AI Now/White/2.0Kg), 83KY001GIN AI Powered Gaming Laptop</t>
         </is>
       </c>
       <c r="C273" t="inlineStr"/>
       <c r="D273" t="n">
-        <v>245490</v>
+        <v>239391</v>
       </c>
       <c r="E273" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
@@ -6172,150 +6172,150 @@
       </c>
       <c r="E274" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 7 FIFA</t>
+          <t>Lenovo Legion Pro 5 2025</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Lenovo Legion Pro 7 FIFA World Cup 26 Edition Intel Core Ultra 9 275HX | NVIDIA RTX 5070Ti 12GB (32GB RAM/1TB SSD/WQXGA OLED/240Hz/16(40.6cm)/Windows 11/Black/2.4Kg), 83F500HPIN AI Gaming Laptop</t>
+          <t>Lenovo Legion Pro 5 2025 AMD Ryzen 9 9955HX | NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/WQXGA OLED/165Hz/16 (40.6cm)/Windows 11/Office 2024+AI Now/Black/2.3Kg), 83F2004CIN AI Powered Gaming Laptop</t>
         </is>
       </c>
       <c r="C275" t="inlineStr"/>
       <c r="D275" t="n">
-        <v>319990</v>
+        <v>245490</v>
       </c>
       <c r="E275" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Lenovo Smartchoice Ideapad 5 2-in-1</t>
+          <t>Lenovo Legion Pro 5 2025</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Lenovo Smartchoice Ideapad 5 2-in-1 13th Gen Intel Core i5-13420H (16GB RAM/512GB SSD/Windows 11/Office Home 2024/WUXGA IPS/14 (35.5cm)/Touchscreen 2-in-1/3Mon.Game Pass/Grey/1.6kg), 83KX0059IN Laptop</t>
+          <t>Lenovo Legion Pro 5 2025 AMD Ryzen 9 9955HX | NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/WQXGA OLED/165Hz/16 (40.6cm)/Windows 11/Office 2024+AI Now/Black/2.3Kg), 83F2004CIN AI Powered Gaming Laptop</t>
         </is>
       </c>
       <c r="C276" t="inlineStr"/>
       <c r="D276" t="n">
-        <v>74490</v>
+        <v>245490</v>
       </c>
       <c r="E276" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Lenovo ThinkBook 15 G5 AMD</t>
+          <t>Lenovo Legion Pro 5 2025</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Lenovo ThinkBook 15 G5 AMD Ryzen 7 7730U 15.6" FHD Antiglare 250 Nits Thin and Light Laptop (8GB RAM/512GB SSD/Windows 11 Home/Fingerprint Reader/Backlit/Mineral Grey/1 Year Onsite/1.7 kg), 21JFA00BIN</t>
+          <t>Lenovo Legion Pro 5 2025 AMD Ryzen 9 9955HX | NVIDIA RTX 5060 8GB (32GB RAM/1TB SSD/WQXGA OLED/165Hz/16 (40.6cm)/Windows 11/Office 2024+AI Now/Black/2.3Kg), 83F2004CIN AI Powered Gaming Laptop</t>
         </is>
       </c>
       <c r="C277" t="inlineStr"/>
       <c r="D277" t="n">
-        <v>59999</v>
+        <v>245490</v>
       </c>
       <c r="E277" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Lenovo ThinkBook 16, Intel Core</t>
+          <t>Lenovo Legion Pro 7 FIFA</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Lenovo ThinkBook 16, Intel Core Ultra 9 185H, 16GB RAM, 512GB SSD, WUXGA IPS 16” (40.64cm), Win 11 Home, Arctic Grey, 1.7Kg, 21SKA0J5IG, Fingerprint, Backlit, 300 Nits, 1Y Warranty, AI Powered Laptop</t>
+          <t>Lenovo Legion Pro 7 FIFA World Cup 26 Edition Intel Core Ultra 9 275HX | NVIDIA RTX 5070Ti 12GB (32GB RAM/1TB SSD/WQXGA OLED/240Hz/16(40.6cm)/Windows 11/Black/2.4Kg), 83F500HPIN AI Gaming Laptop</t>
         </is>
       </c>
       <c r="C278" t="inlineStr"/>
       <c r="D278" t="n">
-        <v>94990</v>
+        <v>319990</v>
       </c>
       <c r="E278" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Lenovo V14 Intel Core i3</t>
+          <t>Lenovo Smartchoice Ideapad 5 2-in-1</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Lenovo V14 Intel Core i3 13th Gen 14" FHD (1920x1080) Antiglare 250 Nits Thin and Light Laptop (16GB RAM/512GB SSD/Windows 11 Home/Office Home 2024/Iron Grey/1.43 kg), 83A0A0PCIN</t>
+          <t>Lenovo Smartchoice Ideapad 5 2-in-1 13th Gen Intel Core i5-13420H (16GB RAM/512GB SSD/Windows 11/Office Home 2024/WUXGA IPS/14 (35.5cm)/Touchscreen 2-in-1/3Mon.Game Pass/Grey/1.6kg), 83KX0059IN Laptop</t>
         </is>
       </c>
       <c r="C279" t="inlineStr"/>
       <c r="D279" t="n">
-        <v>70990</v>
+        <v>74490</v>
       </c>
       <c r="E279" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Lenovo V14 Intel Core i3</t>
+          <t>lenovo_thinkbook_14,_amd_ryzen</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Lenovo V14 Intel Core i3 13th Gen 14" FHD (1920x1080) Antiglare 250 Nits Thin and Light Laptop (16GB RAM/512GB SSD/Windows 11 Home/Office Home 2024/Iron Grey/1.43 kg), 83A0A0PCIN</t>
+          <t>Lenovo ThinkBook 14, AMD Ryzen 5 220, 16GB RAM, 1TB SSD, WUXGA IPS 14” (35.56cm), Windows 11 Home, Arctic Grey, 1.36Kg, 21V0A01SIG, Fingerprint, Backlit, 400 Nits, 1Y Warranty, Laptop</t>
         </is>
       </c>
       <c r="C280" t="inlineStr"/>
       <c r="D280" t="n">
-        <v>70990</v>
+        <v>90990</v>
       </c>
       <c r="E280" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD</t>
+          <t>Lenovo ThinkBook 15 G5 AMD</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
+          <t>Lenovo ThinkBook 15 G5 AMD Ryzen 7 7730U 15.6" FHD Antiglare 250 Nits Thin and Light Laptop (8GB RAM/512GB SSD/Windows 11 Home/Fingerprint Reader/Backlit/Mineral Grey/1 Year Onsite/1.7 kg), 21JFA00BIN</t>
         </is>
       </c>
       <c r="C281" t="inlineStr"/>
       <c r="D281" t="n">
-        <v>44200</v>
+        <v>59999</v>
       </c>
       <c r="E281" t="inlineStr">
         <is>
@@ -6326,231 +6326,231 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD</t>
+          <t>lenovo_thinkbook_16_amd_ryzen</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
+          <t>Lenovo ThinkBook 16 AMD Ryzen 5 7535HS (8GB RAM/512GB SSD/Win 11 Home/Office 2024/Backlit Keyboard/Fingerprint) 16" WUXGA IPS 300 Nits Thin &amp; Light Laptop/1Y Warranty/Aluminium Top/1.7kg, 21MWA0BRIN</t>
         </is>
       </c>
       <c r="C282" t="inlineStr"/>
       <c r="D282" t="n">
-        <v>44490</v>
+        <v>65063</v>
       </c>
       <c r="E282" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD</t>
+          <t>Lenovo ThinkBook 16, Intel Core</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
+          <t>Lenovo ThinkBook 16, Intel Core Ultra 9 185H, 16GB RAM, 512GB SSD, WUXGA IPS 16” (40.64cm), Win 11 Home, Arctic Grey, 1.7Kg, 21SKA0J5IG, Fingerprint, Backlit, 300 Nits, 1Y Warranty, AI Powered Laptop</t>
         </is>
       </c>
       <c r="C283" t="inlineStr"/>
       <c r="D283" t="n">
-        <v>44490</v>
+        <v>94990</v>
       </c>
       <c r="E283" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD</t>
+          <t>Lenovo V14 Intel Core i3</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
+          <t>Lenovo V14 Intel Core i3 13th Gen 14" FHD (1920x1080) Antiglare 250 Nits Thin and Light Laptop (16GB RAM/512GB SSD/Windows 11 Home/Office Home 2024/Iron Grey/1.43 kg), 83A0A0PCIN</t>
         </is>
       </c>
       <c r="C284" t="inlineStr"/>
       <c r="D284" t="n">
-        <v>44500</v>
+        <v>70990</v>
       </c>
       <c r="E284" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD</t>
+          <t>Lenovo V14 Intel Core i3</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
+          <t>Lenovo V14 Intel Core i3 13th Gen 14" FHD (1920x1080) Antiglare 250 Nits Thin and Light Laptop (16GB RAM/512GB SSD/Windows 11 Home/Office Home 2024/Iron Grey/1.43 kg), 83A0A0PCIN</t>
         </is>
       </c>
       <c r="C285" t="inlineStr"/>
       <c r="D285" t="n">
-        <v>49999</v>
+        <v>70990</v>
       </c>
       <c r="E285" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD</t>
+          <t>lenovo_v14_intel_core_i3</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
+          <t>Lenovo V14 Intel Core i3 13th Gen 14" FHD (1920x1080) Antiglare 250 Nits Thin and Light Laptop (16GB RAM/512GB SSD/Windows 11 Home/Office Home 2024/Iron Grey/1.43 kg), 83A0A0PCIN</t>
         </is>
       </c>
       <c r="C286" t="inlineStr"/>
       <c r="D286" t="n">
-        <v>49890</v>
+        <v>70990</v>
       </c>
       <c r="E286" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Lenovo V15 G4 (2024), AMD</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
         </is>
       </c>
       <c r="C287" t="inlineStr"/>
       <c r="D287" t="n">
-        <v>41999</v>
+        <v>44200</v>
       </c>
       <c r="E287" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-22</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Lenovo V15 G4 (2024), AMD</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
         </is>
       </c>
       <c r="C288" t="inlineStr"/>
       <c r="D288" t="n">
-        <v>41999</v>
+        <v>44490</v>
       </c>
       <c r="E288" t="inlineStr">
         <is>
-          <t>2026-05-28</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Lenovo V15 G4 (2024), AMD</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
         </is>
       </c>
       <c r="C289" t="inlineStr"/>
       <c r="D289" t="n">
-        <v>41999</v>
+        <v>44490</v>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Lenovo V15 G4 (2024), AMD</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
         </is>
       </c>
       <c r="C290" t="inlineStr"/>
       <c r="D290" t="n">
-        <v>42999</v>
+        <v>44500</v>
       </c>
       <c r="E290" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Lenovo V15 G4 (2024), AMD</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
         </is>
       </c>
       <c r="C291" t="inlineStr"/>
       <c r="D291" t="n">
-        <v>42999</v>
+        <v>49999</v>
       </c>
       <c r="E291" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon</t>
+          <t>Lenovo V15 G4 (2024), AMD</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
+          <t>Lenovo V15 G4 (2024), AMD Ryzen 3 7320U Quad Core - (8GB/512GB SSD/AMD Radeon Graphics/Windows 11 Home) Thin and Light Business Laptop/15.6" FHD Display/Arctic Grey/1.57 kg/MS Office 2021</t>
         </is>
       </c>
       <c r="C292" t="inlineStr"/>
       <c r="D292" t="n">
-        <v>42999</v>
+        <v>49890</v>
       </c>
       <c r="E292" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
@@ -6567,11 +6567,11 @@
       </c>
       <c r="C293" t="inlineStr"/>
       <c r="D293" t="n">
-        <v>42999</v>
+        <v>41999</v>
       </c>
       <c r="E293" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
@@ -6588,11 +6588,11 @@
       </c>
       <c r="C294" t="inlineStr"/>
       <c r="D294" t="n">
-        <v>42999</v>
+        <v>41999</v>
       </c>
       <c r="E294" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-05-28</t>
         </is>
       </c>
     </row>
@@ -6609,11 +6609,11 @@
       </c>
       <c r="C295" t="inlineStr"/>
       <c r="D295" t="n">
-        <v>44999</v>
+        <v>41999</v>
       </c>
       <c r="E295" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
@@ -6630,11 +6630,11 @@
       </c>
       <c r="C296" t="inlineStr"/>
       <c r="D296" t="n">
-        <v>43999</v>
+        <v>42999</v>
       </c>
       <c r="E296" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
@@ -6651,11 +6651,11 @@
       </c>
       <c r="C297" t="inlineStr"/>
       <c r="D297" t="n">
-        <v>43999</v>
+        <v>42999</v>
       </c>
       <c r="E297" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
@@ -6672,11 +6672,11 @@
       </c>
       <c r="C298" t="inlineStr"/>
       <c r="D298" t="n">
-        <v>43999</v>
+        <v>42999</v>
       </c>
       <c r="E298" t="inlineStr">
         <is>
-          <t>2026-06-11</t>
+          <t>2026-06-03</t>
         </is>
       </c>
     </row>
@@ -6693,11 +6693,11 @@
       </c>
       <c r="C299" t="inlineStr"/>
       <c r="D299" t="n">
-        <v>44999</v>
+        <v>42999</v>
       </c>
       <c r="E299" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
@@ -6714,18 +6714,18 @@
       </c>
       <c r="C300" t="inlineStr"/>
       <c r="D300" t="n">
-        <v>44999</v>
+        <v>42999</v>
       </c>
       <c r="E300" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-06-06</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>lenovo_v15_g4_amd_athlon</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
@@ -6739,133 +6739,133 @@
       </c>
       <c r="E301" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-06-08</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="C302" t="inlineStr"/>
       <c r="D302" t="n">
-        <v>49999</v>
+        <v>43999</v>
       </c>
       <c r="E302" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-06-09</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="C303" t="inlineStr"/>
       <c r="D303" t="n">
-        <v>52760</v>
+        <v>43999</v>
       </c>
       <c r="E303" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-06-10</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="C304" t="inlineStr"/>
       <c r="D304" t="n">
-        <v>52300</v>
+        <v>43999</v>
       </c>
       <c r="E304" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-11</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="C305" t="inlineStr"/>
       <c r="D305" t="n">
-        <v>52490</v>
+        <v>44999</v>
       </c>
       <c r="E305" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-06-12</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen</t>
+          <t>Lenovo V15 G4 AMD Athlon</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="C306" t="inlineStr"/>
       <c r="D306" t="n">
-        <v>52300</v>
+        <v>44999</v>
       </c>
       <c r="E306" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-06-13</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen</t>
+          <t>lenovo_v15_g4_amd_athlon</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
+          <t>Lenovo V15 G4 AMD Athlon Silver 7120U Laptop 8GB LPDDR5 Ram, 512 GB SSD PCIe, Windows 11 Lifetime Validity,15.6" FHD Screen, AMD Radeon 610M, Silver, 1 Year Brand Warranty</t>
         </is>
       </c>
       <c r="C307" t="inlineStr"/>
       <c r="D307" t="n">
-        <v>52890</v>
+        <v>44999</v>
       </c>
       <c r="E307" t="inlineStr">
         <is>
-          <t>2026-05-31</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
@@ -6882,11 +6882,11 @@
       </c>
       <c r="C308" t="inlineStr"/>
       <c r="D308" t="n">
-        <v>53999</v>
+        <v>49999</v>
       </c>
       <c r="E308" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-05-21</t>
         </is>
       </c>
     </row>
@@ -6903,11 +6903,11 @@
       </c>
       <c r="C309" t="inlineStr"/>
       <c r="D309" t="n">
-        <v>53999</v>
+        <v>52760</v>
       </c>
       <c r="E309" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-05-24</t>
         </is>
       </c>
     </row>
@@ -6924,322 +6924,322 @@
       </c>
       <c r="C310" t="inlineStr"/>
       <c r="D310" t="n">
-        <v>54790</v>
+        <v>52300</v>
       </c>
       <c r="E310" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>lenovo_v15_g6_amd_ryzen</t>
+          <t>Lenovo V15 G4 AMD Ryzen</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Lenovo V15 G6 AMD Ryzen 7 170 (Coequal 7735HS) 15.6" (39.62cm) FHD Thin and Light Business Laptop (16GB RAM DDR5/ 512GB SSD/Windows 11/ MS Office 2024/ AMD Radeon Graphics/Luna Grey/ 1.6 kg)</t>
+          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
         </is>
       </c>
       <c r="C311" t="inlineStr"/>
       <c r="D311" t="n">
-        <v>64999</v>
+        <v>52490</v>
       </c>
       <c r="E311" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-05-26</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7 (Smartchoice)</t>
+          <t>Lenovo V15 G4 AMD Ryzen</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7 (Smartchoice) Aura Edition, Intel Core Ultra 5 226V, 16GB RAM, 1TB SSD, WUXGA OLED, Copilot+ AI PC, 40 TOPS, 14"/35.5cm, Windows 11, Office 2024, Grey, 1.19Kg, 83JX005FIN, AI Laptop</t>
+          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
         </is>
       </c>
       <c r="C312" t="inlineStr"/>
       <c r="D312" t="n">
-        <v>99990</v>
+        <v>52300</v>
       </c>
       <c r="E312" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-27</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7 (Smartchoice)</t>
+          <t>Lenovo V15 G4 AMD Ryzen</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7 (Smartchoice) Aura Edition, Intel Core Ultra 5 226V, 16GB RAM, 1TB SSD, WUXGA OLED, Copilot+ AI PC, 40 TOPS, 14"/35.5cm, Windows 11, Office 2024, Grey, 1.19Kg, 83JX005FIN, AI Laptop</t>
+          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
         </is>
       </c>
       <c r="C313" t="inlineStr"/>
       <c r="D313" t="n">
-        <v>105939</v>
+        <v>52890</v>
       </c>
       <c r="E313" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-31</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7, Intel</t>
+          <t>Lenovo V15 G4 AMD Ryzen</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7, Intel Core Ultra 5 125H, 16GB RAM, 512GB SSD, AI PC, WUXGA-OLED, 14"/35.5cm, Windows 11, Microsoft 365 Basic + Office 2024, Grey, 1.39Kg, 83CV00DFIN, AI Powered Laptop</t>
+          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
         </is>
       </c>
       <c r="C314" t="inlineStr"/>
       <c r="D314" t="n">
-        <v>77990</v>
+        <v>53999</v>
       </c>
       <c r="E314" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-06-01</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7, Intel</t>
+          <t>Lenovo V15 G4 AMD Ryzen</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Lenovo Yoga Slim 7, Intel Core Ultra 5 125H, 16GB RAM, 512GB SSD, AI PC, WUXGA-OLED, 14"/35.5cm, Windows 11, Microsoft 365 Basic + Office 2024, Grey, 1.39Kg, 83CV00DFIN, AI Powered Laptop</t>
+          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
         </is>
       </c>
       <c r="C315" t="inlineStr"/>
       <c r="D315" t="n">
-        <v>84990</v>
+        <v>53999</v>
       </c>
       <c r="E315" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-02</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Lenovo {SmartChoice Chromebook, Intel Celeron</t>
+          <t>Lenovo V15 G4 AMD Ryzen</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Lenovo {SmartChoice Chromebook, Intel Celeron N4500, 4GB RAM, 64GB eMMC, HD, 11.6"/29.46cm, Chrome OS, Blue, 1.21Kg, 2Wx2 Stereo Speakers, HD Camera, 82UY0014HA, Laptop</t>
+          <t>Lenovo V15 G4 AMD Ryzen 5 7520U 15.6 inch FHD Laptop, AMD Graphics, 16GB DDR5 5500Mhz Ram, 512GB SSD NVMe, Windows 11, Dolby Audio, Arctic Grey, 1 Year Onsite Brand Warranty</t>
         </is>
       </c>
       <c r="C316" t="inlineStr"/>
       <c r="D316" t="n">
-        <v>21990</v>
+        <v>54790</v>
       </c>
       <c r="E316" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Lenovo {SmartChoice Chromebook, Intel Celeron</t>
+          <t>lenovo_v15_g6_amd_ryzen</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Lenovo {SmartChoice Chromebook, Intel Celeron N4500, 4GB RAM, 64GB eMMC, HD, 11.6"/29.46cm, Chrome OS, Blue, 1.21Kg, 2Wx2 Stereo Speakers, HD Camera, 82UY0014HA, Laptop</t>
+          <t>Lenovo V15 G6 AMD Ryzen 7 170 (Coequal 7735HS) 15.6" (39.62cm) FHD Thin and Light Business Laptop (16GB RAM DDR5/ 512GB SSD/Windows 11/ MS Office 2024/ AMD Radeon Graphics/Luna Grey/ 1.6 kg)</t>
         </is>
       </c>
       <c r="C317" t="inlineStr"/>
       <c r="D317" t="n">
-        <v>17990</v>
+        <v>64999</v>
       </c>
       <c r="E317" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Samsung Galaxy Book6 (Gray, 16GB</t>
+          <t>Lenovo Yoga Slim 7 (Smartchoice)</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Samsung Galaxy Book6 (Gray, 16GB RAM, 1TB SSD) | Intel Core Ultra 5 (Series 3) | 16" WUXGA+ Display with Touchscreen | 24Hrs Battery Life | 120 Hz Refresh Rate | Dolby Atmos Stereo Speakers | AI PC</t>
+          <t>Lenovo Yoga Slim 7 (Smartchoice) Aura Edition, Intel Core Ultra 5 226V, 16GB RAM, 1TB SSD, WUXGA OLED, Copilot+ AI PC, 40 TOPS, 14"/35.5cm, Windows 11, Office 2024, Grey, 1.19Kg, 83JX005FIN, AI Laptop</t>
         </is>
       </c>
       <c r="C318" t="inlineStr"/>
       <c r="D318" t="n">
-        <v>146990</v>
+        <v>99990</v>
       </c>
       <c r="E318" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C</t>
+          <t>Lenovo Yoga Slim 7 (Smartchoice)</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
+          <t>Lenovo Yoga Slim 7 (Smartchoice) Aura Edition, Intel Core Ultra 5 226V, 16GB RAM, 1TB SSD, WUXGA OLED, Copilot+ AI PC, 40 TOPS, 14"/35.5cm, Windows 11, Office 2024, Grey, 1.19Kg, 83JX005FIN, AI Laptop</t>
         </is>
       </c>
       <c r="C319" t="inlineStr"/>
       <c r="D319" t="n">
-        <v>12990</v>
+        <v>105939</v>
       </c>
       <c r="E319" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C</t>
+          <t>Lenovo Yoga Slim 7, Intel</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
+          <t>Lenovo Yoga Slim 7, Intel Core Ultra 5 125H, 16GB RAM, 512GB SSD, AI PC, WUXGA-OLED, 14"/35.5cm, Windows 11, Microsoft 365 Basic + Office 2024, Grey, 1.39Kg, 83CV00DFIN, AI Powered Laptop</t>
         </is>
       </c>
       <c r="C320" t="inlineStr"/>
       <c r="D320" t="n">
-        <v>12990</v>
+        <v>77990</v>
       </c>
       <c r="E320" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C</t>
+          <t>Lenovo Yoga Slim 7, Intel</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
+          <t>Lenovo Yoga Slim 7, Intel Core Ultra 5 125H, 16GB RAM, 512GB SSD, AI PC, WUXGA-OLED, 14"/35.5cm, Windows 11, Microsoft 365 Basic + Office 2024, Grey, 1.39Kg, 83CV00DFIN, AI Powered Laptop</t>
         </is>
       </c>
       <c r="C321" t="inlineStr"/>
       <c r="D321" t="n">
-        <v>22990</v>
+        <v>84990</v>
       </c>
       <c r="E321" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-19</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C</t>
+          <t>Lenovo {SmartChoice Chromebook, Intel Celeron</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
+          <t>Lenovo {SmartChoice Chromebook, Intel Celeron N4500, 4GB RAM, 64GB eMMC, HD, 11.6"/29.46cm, Chrome OS, Blue, 1.21Kg, 2Wx2 Stereo Speakers, HD Camera, 82UY0014HA, Laptop</t>
         </is>
       </c>
       <c r="C322" t="inlineStr"/>
       <c r="D322" t="n">
-        <v>22990</v>
+        <v>21990</v>
       </c>
       <c r="E322" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>acer Aspire 3, Intel Core</t>
+          <t>Lenovo {SmartChoice Chromebook, Intel Celeron</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>acer Aspire 3, Intel Core Celeron N4500, 12GB LPDDR4X RAM, 512GB SSD, HD, 15.6"/39.62cm, Windows 11 Home, Pure Silver, 1.5KG, A325-45, Thin and Light Laptop</t>
+          <t>Lenovo {SmartChoice Chromebook, Intel Celeron N4500, 4GB RAM, 64GB eMMC, HD, 11.6"/29.46cm, Chrome OS, Blue, 1.21Kg, 2Wx2 Stereo Speakers, HD Camera, 82UY0014HA, Laptop</t>
         </is>
       </c>
       <c r="C323" t="inlineStr"/>
       <c r="D323" t="n">
-        <v>39890</v>
+        <v>17990</v>
       </c>
       <c r="E323" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>acer Aspire Lite, AMD Ryzen</t>
+          <t>primebook_2_max_(2026)_|</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>acer Aspire Lite, AMD Ryzen 3 5300U Processor, 16 GB RAM, 512GB SSD, Full HD, 15.6"/39.62cm, Windows 11 Home, Steel Gray, 1.59KG, AL15-41, Metal Body, Premium Thin and Light Laptop</t>
+          <t>Primebook 2 Max (2026) | 8GB RAM, 256GB UFS Storage | 15.6-Inch Full HD IPS Display | 12hrs Battery | MediaTek Helio G99 | Android 15 (PrimeOS 3.0) | Backlit Keyboard | in-Built AI (Gray)</t>
         </is>
       </c>
       <c r="C324" t="inlineStr"/>
       <c r="D324" t="n">
-        <v>42990</v>
+        <v>29990</v>
       </c>
       <c r="E324" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>Samsung Galaxy Book6 (Gray, 16GB</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>Samsung Galaxy Book6 (Gray, 16GB RAM, 1TB SSD) | Intel Core Ultra 5 (Series 3) | 16" WUXGA+ Display with Touchscreen | 24Hrs Battery Life | 120 Hz Refresh Rate | Dolby Atmos Stereo Speakers | AI PC</t>
         </is>
       </c>
       <c r="C325" t="inlineStr"/>
       <c r="D325" t="n">
-        <v>45990</v>
+        <v>146990</v>
       </c>
       <c r="E325" t="inlineStr">
         <is>
@@ -7250,59 +7250,59 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
         </is>
       </c>
       <c r="C326" t="inlineStr"/>
       <c r="D326" t="n">
-        <v>45990</v>
+        <v>12990</v>
       </c>
       <c r="E326" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
         </is>
       </c>
       <c r="C327" t="inlineStr"/>
       <c r="D327" t="n">
-        <v>45990</v>
+        <v>12990</v>
       </c>
       <c r="E327" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-23</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
         </is>
       </c>
       <c r="C328" t="inlineStr"/>
       <c r="D328" t="n">
-        <v>43990</v>
+        <v>22990</v>
       </c>
       <c r="E328" t="inlineStr">
         <is>
@@ -7313,63 +7313,63 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>Thomson NEO 14.1 Inch IN-P14C Intel Celeron Dual Core N4020 Processor &amp; Window 11 Home Notebook (4 GB RAM DDR4/ 128 GB SSD/Numeric Touch Pad/Thin &amp; Light Weight/Silver)</t>
         </is>
       </c>
       <c r="C329" t="inlineStr"/>
       <c r="D329" t="n">
-        <v>43990</v>
+        <v>22990</v>
       </c>
       <c r="E329" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>acer Aspire 3, Intel Core</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>acer Aspire 3, Intel Core Celeron N4500, 12GB LPDDR4X RAM, 512GB SSD, HD, 15.6"/39.62cm, Windows 11 Home, Pure Silver, 1.5KG, A325-45, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C330" t="inlineStr"/>
       <c r="D330" t="n">
-        <v>43990</v>
+        <v>39890</v>
       </c>
       <c r="E330" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD</t>
+          <t>acer Aspire Lite, AMD Ryzen</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
+          <t>acer Aspire Lite, AMD Ryzen 3 5300U Processor, 16 GB RAM, 512GB SSD, Full HD, 15.6"/39.62cm, Windows 11 Home, Steel Gray, 1.59KG, AL15-41, Metal Body, Premium Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C331" t="inlineStr"/>
       <c r="D331" t="n">
-        <v>43990</v>
+        <v>42990</v>
       </c>
       <c r="E331" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
@@ -7386,238 +7386,238 @@
       </c>
       <c r="C332" t="inlineStr"/>
       <c r="D332" t="n">
-        <v>43990</v>
+        <v>45990</v>
       </c>
       <c r="E332" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-04-15</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop ModeI 7410 Laptop |</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop ModeI 7410 Laptop | InteI Core i5 10th Gen | 16GB DDR4 RAM | 256GB SSD | 14" Full HD Display | Win 10 Pro | InteI UHD Graphics 620 | 3 Months Seller Warranty | A+ Condition (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C333" t="inlineStr"/>
       <c r="D333" t="n">
-        <v>27299</v>
+        <v>45990</v>
       </c>
       <c r="E333" t="inlineStr">
         <is>
-          <t>2026-04-25</t>
+          <t>2026-04-16</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C334" t="inlineStr"/>
       <c r="D334" t="n">
-        <v>26999</v>
+        <v>45990</v>
       </c>
       <c r="E334" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C335" t="inlineStr"/>
       <c r="D335" t="n">
-        <v>26400</v>
+        <v>43990</v>
       </c>
       <c r="E335" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-08</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C336" t="inlineStr"/>
       <c r="D336" t="n">
-        <v>28599</v>
+        <v>43990</v>
       </c>
       <c r="E336" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
+          <t>2026-05-09</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C337" t="inlineStr"/>
       <c r="D337" t="n">
-        <v>28999</v>
+        <v>43990</v>
       </c>
       <c r="E337" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C338" t="inlineStr"/>
       <c r="D338" t="n">
-        <v>31990</v>
+        <v>43990</v>
       </c>
       <c r="E338" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-05-14</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>acer SmartChoice Aspire Lite, AMD</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>acer SmartChoice Aspire Lite, AMD Ryzen 5-5625U Processor, 16 GB/512 GB, Full HD, 15.6"/39.62 cm, Windows 11 Home, Steel Gray, 1.59 kg, AL15-41, Metal Body, Thin and Light Laptop</t>
         </is>
       </c>
       <c r="C339" t="inlineStr"/>
       <c r="D339" t="n">
-        <v>35490</v>
+        <v>43990</v>
       </c>
       <c r="E339" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-05-15</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+          <t>𝗗𝗲𝗹𝗹Laptop ModeI 7410 Laptop |</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+          <t>𝗗𝗲𝗹𝗹Laptop ModeI 7410 Laptop | InteI Core i5 10th Gen | 16GB DDR4 RAM | 256GB SSD | 14" Full HD Display | Win 10 Pro | InteI UHD Graphics 620 | 3 Months Seller Warranty | A+ Condition (Refab)</t>
         </is>
       </c>
       <c r="C340" t="inlineStr"/>
       <c r="D340" t="n">
-        <v>37490</v>
+        <v>27299</v>
       </c>
       <c r="E340" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-04-25</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Model E5570 Laptop | Core</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>𝗗𝗲𝗹𝗹Model E5570 Laptop | Core i7 6th Gen | 8GB Fast RAM | 256GB SSD | 15.6" HD Display | HD Graphics | Win 10 | WiFi| (Pre-Owned &amp; Tested)</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
         </is>
       </c>
       <c r="C341" t="inlineStr"/>
       <c r="D341" t="n">
-        <v>20599</v>
+        <v>26999</v>
       </c>
       <c r="E341" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-10</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop | InteI i5 6th Gen | 8GB RAM | 256GB SSD | WiFi | Webcam | Win10 Pro (Refab)</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
         </is>
       </c>
       <c r="C342" t="inlineStr"/>
       <c r="D342" t="n">
-        <v>20299</v>
+        <v>26400</v>
       </c>
       <c r="E342" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-20</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop | 𝗜𝗡𝗧𝗘𝗟i5 6th Gen | 8GB RAM | 256GB SSD | WiFi | Webcam | Win10 Pro (Refab)</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
         </is>
       </c>
       <c r="C343" t="inlineStr"/>
       <c r="D343" t="n">
-        <v>20499</v>
+        <v>28599</v>
       </c>
       <c r="E343" t="inlineStr">
         <is>
@@ -7628,21 +7628,189 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop | 𝗜𝗡𝗧𝗘𝗟i5 6th Gen | 8GB RAM | 256GB SSD | WiFi | Webcam | Win10 Pro (Refab)</t>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
         </is>
       </c>
       <c r="C344" t="inlineStr"/>
       <c r="D344" t="n">
+        <v>28999</v>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr"/>
+      <c r="D345" t="n">
+        <v>31990</v>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>2026-06-03</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr"/>
+      <c r="D346" t="n">
+        <v>35490</v>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Laptop Model 5420 | 𝗜𝗡𝗧𝗘𝗟i5 11th Gen Processor |8GB DDR4 RAM |256GB SSD |14" FHD Display | Win10 | A+ Condition Laptop (Refab)</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr"/>
+      <c r="D347" t="n">
+        <v>37490</v>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>2026-06-08</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Model E5570 Laptop | Core</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>𝗗𝗲𝗹𝗹Model E5570 Laptop | Core i7 6th Gen | 8GB Fast RAM | 256GB SSD | 15.6" HD Display | HD Graphics | Win 10 | WiFi| (Pre-Owned &amp; Tested)</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr"/>
+      <c r="D348" t="n">
+        <v>20599</v>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>2026-05-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop | InteI i5 6th Gen | 8GB RAM | 256GB SSD | WiFi | Webcam | Win10 Pro (Refab)</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr"/>
+      <c r="D349" t="n">
+        <v>20299</v>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop | 𝗜𝗡𝗧𝗘𝗟i5 6th Gen | 8GB RAM | 256GB SSD | WiFi | Webcam | Win10 Pro (Refab)</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr"/>
+      <c r="D350" t="n">
+        <v>20499</v>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>𝗛𝗣𝗣𝗿𝗼𝗯𝗼𝗼𝗸Model 430 G3 Business Laptop | 𝗜𝗡𝗧𝗘𝗟i5 6th Gen | 8GB RAM | 256GB SSD | WiFi | Webcam | Win10 Pro (Refab)</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr"/>
+      <c r="D351" t="n">
         <v>19999</v>
       </c>
-      <c r="E344" t="inlineStr">
+      <c r="E351" t="inlineStr">
         <is>
           <t>2026-05-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>𝗟𝗲𝗻𝗼𝘃𝗼model_l14_laptop|_core_i5</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>𝗟𝗲𝗻𝗼𝘃𝗼Model L14 Laptop| Core i5 11th Gen Processor | 16GB Fast RAM/ 256GB SSD | 14″ HD Display | A+ (Pre-Owned &amp; Tested)</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr"/>
+      <c r="D352" t="n">
+        <v>31599</v>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>2026-07-21</t>
         </is>
       </c>
     </row>

</xml_diff>